<commit_message>
Revidovat kapitolu 3 po posouzeni
Sjednotit nazvoslovi (1. a 3. kvartil, spicatost, chvost, velikost vyberu),
opravit vecne a didakticke nepresnosti vykladu, doplnit cviceni 8 a 12,
presunout data prikladu do sesitu a zrusit CSV. Zaznam R14 a autorska historie.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kapitola_03.xlsx
+++ b/data/kapitola_03.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\R Projects\github\statistics-for-psychology\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F9FA881-4D42-49E3-A01B-0EB3EF2D7F60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5BF2A6A-774E-4062-BEA4-19E5A5917DE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-109" yWindow="-109" windowWidth="34995" windowHeight="19060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,8 @@
     <sheet name="Priklad" sheetId="1" r:id="rId1"/>
     <sheet name="Souhrn" sheetId="2" r:id="rId2"/>
     <sheet name="Rozsireni" sheetId="3" r:id="rId3"/>
-    <sheet name="Data" sheetId="4" r:id="rId4"/>
+    <sheet name="Dalsi_priklady" sheetId="5" r:id="rId4"/>
+    <sheet name="Data" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="137">
   <si>
     <t>Doba (min)</t>
   </si>
@@ -83,15 +84,9 @@
     <t>Maximum (min)</t>
   </si>
   <si>
-    <t>Dolní kvartil (min)</t>
-  </si>
-  <si>
     <t>Autorský příklad: pět vyplněných číselných časů. Žluté buňky jsou vstupy, modré vzorce.</t>
   </si>
   <si>
-    <t>Horní kvartil (min)</t>
-  </si>
-  <si>
     <t>Variační rozpětí (min)</t>
   </si>
   <si>
@@ -170,24 +165,15 @@
     <t>Nejvyšší hodnota</t>
   </si>
   <si>
-    <t>Dolní kvartil</t>
-  </si>
-  <si>
     <t>Interpolace při podílu 0,25</t>
   </si>
   <si>
-    <t>Horní kvartil</t>
-  </si>
-  <si>
     <t>Interpolace při podílu 0,75</t>
   </si>
   <si>
     <t>Mezikvartilové rozpětí</t>
   </si>
   <si>
-    <t>Horní minus dolní kvartil</t>
-  </si>
-  <si>
     <t>Výběrový rozptyl</t>
   </si>
   <si>
@@ -408,6 +394,60 @@
   </si>
   <si>
     <t>P36</t>
+  </si>
+  <si>
+    <t>1. kvartil (min)</t>
+  </si>
+  <si>
+    <t>3. kvartil (min)</t>
+  </si>
+  <si>
+    <t>1. kvartil</t>
+  </si>
+  <si>
+    <t>3. kvartil</t>
+  </si>
+  <si>
+    <t>3. kvartil minus 1. kvartil</t>
+  </si>
+  <si>
+    <t>SKEW.P a SKEW používají různé konvence. KURT vrací korigovaný exces, nikoli špičatost před odečtením tří.</t>
+  </si>
+  <si>
+    <t>Doby pro kvantily (min)</t>
+  </si>
+  <si>
+    <t>Doby pro ořezání (min)</t>
+  </si>
+  <si>
+    <t>Skóry pro krabicový graf (body)</t>
+  </si>
+  <si>
+    <t>17. percentil jedenácti dob (min)</t>
+  </si>
+  <si>
+    <t>Průměr deseti dob (min)</t>
+  </si>
+  <si>
+    <t>Medián deseti dob (min)</t>
+  </si>
+  <si>
+    <t>1. kvartil skórů (body)</t>
+  </si>
+  <si>
+    <t>Medián skórů (body)</t>
+  </si>
+  <si>
+    <t>3. kvartil skórů (body)</t>
+  </si>
+  <si>
+    <t>Mezikvartilové rozpětí skórů (body)</t>
+  </si>
+  <si>
+    <t>Autorské modelové údaje z výkladu kapitoly. Nejde o skutečný výzkum.</t>
+  </si>
+  <si>
+    <t>Ořezání a winsorizaci proveďte podle výkladu ručně; sešit je záměrně nepočítá.</t>
   </si>
 </sst>
 </file>
@@ -418,7 +458,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -443,8 +483,30 @@
       <sz val="11"/>
       <name val="Carlito"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF223744"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF526775"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -466,6 +528,24 @@
         <fgColor rgb="FFEAF4F8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF234F62"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF1CB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEAF4F8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -480,7 +560,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -509,14 +589,29 @@
     <xf numFmtId="165" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -982,7 +1077,7 @@
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
       <c r="I8" s="6" t="s">
-        <v>15</v>
+        <v>119</v>
       </c>
       <c r="J8" s="5">
         <f>_xlfn.PERCENTILE.INC(A2:A6,0.25)</f>
@@ -990,30 +1085,30 @@
       </c>
     </row>
     <row r="9" spans="1:10" ht="36" customHeight="1">
-      <c r="A9" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="F9" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>16</v>
+      <c r="A9" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="G9" s="15" t="s">
+        <v>15</v>
       </c>
       <c r="H9" s="6"/>
       <c r="I9" s="6" t="s">
-        <v>17</v>
+        <v>120</v>
       </c>
       <c r="J9" s="5">
         <f>_xlfn.PERCENTILE.INC(A2:A6,0.75)</f>
@@ -1030,7 +1125,7 @@
       <c r="G10" s="6"/>
       <c r="H10" s="6"/>
       <c r="I10" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="J10" s="5">
         <f>J7-J6</f>
@@ -1038,30 +1133,30 @@
       </c>
     </row>
     <row r="11" spans="1:10" ht="36" customHeight="1">
-      <c r="A11" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="F11" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>19</v>
+      <c r="A11" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G11" s="15" t="s">
+        <v>17</v>
       </c>
       <c r="H11" s="6"/>
       <c r="I11" s="6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="J11" s="5">
         <f>J9-J8</f>
@@ -1078,7 +1173,7 @@
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
       <c r="I12" s="6" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="J12" s="5">
         <f>AVERAGE(C2:C6)</f>
@@ -1086,30 +1181,30 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="36" customHeight="1">
-      <c r="A13" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="F13" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>22</v>
+      <c r="A13" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="F13" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="G13" s="15" t="s">
+        <v>20</v>
       </c>
       <c r="H13" s="6"/>
       <c r="I13" s="6" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="J13" s="5">
         <f>SUM(D2:D6)</f>
@@ -1126,7 +1221,7 @@
       <c r="G14" s="6"/>
       <c r="H14" s="6"/>
       <c r="I14" s="6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J14" s="5">
         <f>J13/J2</f>
@@ -1134,30 +1229,30 @@
       </c>
     </row>
     <row r="15" spans="1:10" ht="36" customHeight="1">
-      <c r="A15" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="E15" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="F15" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="G15" s="10" t="s">
-        <v>25</v>
+      <c r="A15" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="E15" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F15" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="G15" s="15" t="s">
+        <v>23</v>
       </c>
       <c r="H15" s="6"/>
       <c r="I15" s="6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J15" s="5">
         <f>_xlfn.VAR.S(A2:A6)</f>
@@ -1174,7 +1269,7 @@
       <c r="G16" s="6"/>
       <c r="H16" s="6"/>
       <c r="I16" s="6" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="J16" s="5">
         <f>_xlfn.STDEV.S(A2:A6)</f>
@@ -1191,7 +1286,7 @@
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
       <c r="I17" s="6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="J17" s="5">
         <f>MEDIAN(E2:E6)</f>
@@ -1211,35 +1306,35 @@
       <c r="J18" s="1"/>
     </row>
     <row r="19" spans="1:10" ht="36" customHeight="1">
-      <c r="A19" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="C19" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="D19" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="E19" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="F19" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="G19" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="H19" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="I19" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="J19" s="11" t="s">
-        <v>29</v>
+      <c r="A19" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="D19" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="F19" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="G19" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="H19" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="I19" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="J19" s="14" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="22.95" customHeight="1">
@@ -1255,35 +1350,35 @@
       <c r="J20" s="1"/>
     </row>
     <row r="21" spans="1:10" ht="36" customHeight="1">
-      <c r="A21" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="B21" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="C21" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="D21" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="E21" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="F21" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="G21" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="H21" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="I21" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="J21" s="11" t="s">
-        <v>30</v>
+      <c r="A21" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="F21" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="H21" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="I21" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="J21" s="14" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="22.95" customHeight="1">
@@ -1543,13 +1638,13 @@
         <v>7</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>33</v>
       </c>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
@@ -1560,7 +1655,7 @@
     </row>
     <row r="2" spans="1:10" ht="22.95" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B2" s="7">
         <f>COUNT(Data!B2:B37)</f>
@@ -1571,7 +1666,7 @@
         <v>36</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
@@ -1582,7 +1677,7 @@
     </row>
     <row r="3" spans="1:10" ht="22.95" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B3" s="5">
         <f>AVERAGE(Data!B2:B37)</f>
@@ -1593,7 +1688,7 @@
         <v>7.0277777777777777</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -1604,7 +1699,7 @@
     </row>
     <row r="4" spans="1:10" ht="22.95" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B4" s="5">
         <f>MEDIAN(Data!B2:B37)</f>
@@ -1615,7 +1710,7 @@
         <v>7</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
@@ -1626,7 +1721,7 @@
     </row>
     <row r="5" spans="1:10" ht="22.95" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B5" s="5">
         <f>MIN(Data!B2:B37)</f>
@@ -1637,7 +1732,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -1648,7 +1743,7 @@
     </row>
     <row r="6" spans="1:10" ht="22.95" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B6" s="5">
         <f>MAX(Data!B2:B37)</f>
@@ -1659,7 +1754,7 @@
         <v>12</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
@@ -1670,7 +1765,7 @@
     </row>
     <row r="7" spans="1:10" ht="22.95" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>44</v>
+        <v>121</v>
       </c>
       <c r="B7" s="5">
         <f>_xlfn.PERCENTILE.INC(Data!B2:B37,0.25)</f>
@@ -1681,7 +1776,7 @@
         <v>5.75</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -1692,7 +1787,7 @@
     </row>
     <row r="8" spans="1:10" ht="22.95" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>46</v>
+        <v>122</v>
       </c>
       <c r="B8" s="5">
         <f>_xlfn.PERCENTILE.INC(Data!B2:B37,0.75)</f>
@@ -1703,7 +1798,7 @@
         <v>9</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
@@ -1714,7 +1809,7 @@
     </row>
     <row r="9" spans="1:10" ht="22.95" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B9" s="5">
         <f>B8-B7</f>
@@ -1725,7 +1820,7 @@
         <v>3.25</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>49</v>
+        <v>123</v>
       </c>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
@@ -1736,7 +1831,7 @@
     </row>
     <row r="10" spans="1:10" ht="22.95" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B10" s="5">
         <f>_xlfn.VAR.S(Data!B2:B37)</f>
@@ -1747,7 +1842,7 @@
         <v>6.7134920634920618</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
@@ -1758,7 +1853,7 @@
     </row>
     <row r="11" spans="1:10" ht="22.95" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B11" s="5">
         <f>_xlfn.STDEV.S(Data!B2:B37)</f>
@@ -1769,7 +1864,7 @@
         <v>2.5910407298018421</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
@@ -1803,17 +1898,17 @@
       <c r="J13" s="1"/>
     </row>
     <row r="14" spans="1:10" ht="36" customHeight="1">
-      <c r="A14" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>54</v>
+      <c r="A14" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>49</v>
       </c>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
@@ -1835,17 +1930,17 @@
       <c r="J15" s="1"/>
     </row>
     <row r="16" spans="1:10" ht="36" customHeight="1">
-      <c r="A16" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="C16" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="D16" s="11" t="s">
-        <v>55</v>
+      <c r="A16" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>50</v>
       </c>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
@@ -2165,23 +2260,23 @@
   <sheetData>
     <row r="1" spans="1:10" ht="44" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="2" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>8</v>
@@ -2189,7 +2284,7 @@
     </row>
     <row r="2" spans="1:10" ht="22.95" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="B2" s="3">
         <v>4</v>
@@ -2207,7 +2302,7 @@
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="J2" s="5">
         <f>AVERAGE(Priklad!F2:F6)/(SQRT(Priklad!J14)^3)</f>
@@ -2216,7 +2311,7 @@
     </row>
     <row r="3" spans="1:10" ht="22.95" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="B3" s="3">
         <v>2</v>
@@ -2234,7 +2329,7 @@
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
       <c r="I3" s="1" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="J3" s="5">
         <f>_xlfn.SKEW.P(Priklad!A2:A6)</f>
@@ -2243,7 +2338,7 @@
     </row>
     <row r="4" spans="1:10" ht="22.95" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="B4" s="3">
         <v>2</v>
@@ -2261,7 +2356,7 @@
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
       <c r="I4" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="J4" s="5">
         <f>SKEW(Priklad!A2:A6)</f>
@@ -2270,7 +2365,7 @@
     </row>
     <row r="5" spans="1:10" ht="22.95" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="B5" s="3">
         <v>0</v>
@@ -2288,7 +2383,7 @@
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
       <c r="I5" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="J5" s="5">
         <f>AVERAGE(Priklad!G2:G6)/(Priklad!J14^2)-3</f>
@@ -2305,7 +2400,7 @@
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
       <c r="I6" s="1" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="J6" s="5">
         <f>KURT(Priklad!A2:A6)</f>
@@ -2313,11 +2408,11 @@
       </c>
     </row>
     <row r="7" spans="1:10" ht="22.95" customHeight="1">
-      <c r="A7" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
+      <c r="A7" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
       <c r="D7" s="5">
         <f>SUM(D2:D5)</f>
         <v>1.5</v>
@@ -2354,35 +2449,35 @@
       <c r="J9" s="1"/>
     </row>
     <row r="10" spans="1:10" ht="36" customHeight="1">
-      <c r="A10" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="E10" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="F10" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="G10" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="H10" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="I10" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="J10" s="11" t="s">
-        <v>71</v>
+      <c r="A10" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="F10" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="G10" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="H10" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="I10" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="J10" s="14" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="22.95" customHeight="1">
@@ -2398,35 +2493,35 @@
       <c r="J11" s="1"/>
     </row>
     <row r="12" spans="1:10" ht="36" customHeight="1">
-      <c r="A12" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="E12" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="F12" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="G12" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="H12" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="I12" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="J12" s="11" t="s">
-        <v>72</v>
+      <c r="A12" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="F12" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="G12" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="H12" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="I12" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="J12" s="14" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="22.95" customHeight="1">
@@ -2442,35 +2537,35 @@
       <c r="J13" s="1"/>
     </row>
     <row r="14" spans="1:10" ht="36" customHeight="1">
-      <c r="A14" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="F14" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="G14" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="H14" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="I14" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="J14" s="11" t="s">
-        <v>73</v>
+      <c r="A14" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="F14" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="G14" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="H14" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="J14" s="14" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="22.95" customHeight="1">
@@ -2802,6 +2897,743 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{110165F7-3E83-4FCA-9326-82EB28C77487}">
+  <dimension ref="A1:J45"/>
+  <sheetFormatPr defaultRowHeight="13.6"/>
+  <cols>
+    <col min="1" max="1" width="18.77734375" customWidth="1"/>
+    <col min="2" max="2" width="3.77734375" customWidth="1"/>
+    <col min="3" max="3" width="18.77734375" customWidth="1"/>
+    <col min="4" max="4" width="3.77734375" customWidth="1"/>
+    <col min="5" max="5" width="22.77734375" customWidth="1"/>
+    <col min="6" max="6" width="3.77734375" customWidth="1"/>
+    <col min="7" max="7" width="38.77734375" customWidth="1"/>
+    <col min="8" max="8" width="14.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="44" customHeight="1">
+      <c r="A1" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="B1" s="10"/>
+      <c r="C1" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="D1" s="10"/>
+      <c r="E1" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="F1" s="10"/>
+      <c r="G1" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+    </row>
+    <row r="2" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A2" s="12">
+        <v>4</v>
+      </c>
+      <c r="B2" s="10"/>
+      <c r="C2" s="12">
+        <v>2</v>
+      </c>
+      <c r="D2" s="10"/>
+      <c r="E2" s="12">
+        <v>2</v>
+      </c>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="H2" s="13">
+        <f>_xlfn.PERCENTILE.INC(A2:A12,0.17)</f>
+        <v>6.4</v>
+      </c>
+      <c r="I2" s="10"/>
+      <c r="J2" s="10"/>
+    </row>
+    <row r="3" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A3" s="12">
+        <v>5</v>
+      </c>
+      <c r="B3" s="10"/>
+      <c r="C3" s="12">
+        <v>3</v>
+      </c>
+      <c r="D3" s="10"/>
+      <c r="E3" s="12">
+        <v>5</v>
+      </c>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="H3" s="13">
+        <f>AVERAGE(C2:C11)</f>
+        <v>8</v>
+      </c>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+    </row>
+    <row r="4" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A4" s="12">
+        <v>7</v>
+      </c>
+      <c r="B4" s="10"/>
+      <c r="C4" s="12">
+        <v>4</v>
+      </c>
+      <c r="D4" s="10"/>
+      <c r="E4" s="12">
+        <v>15</v>
+      </c>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="H4" s="13">
+        <f>MEDIAN(C2:C11)</f>
+        <v>5.5</v>
+      </c>
+      <c r="I4" s="10"/>
+      <c r="J4" s="10"/>
+    </row>
+    <row r="5" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A5" s="12">
+        <v>8</v>
+      </c>
+      <c r="B5" s="10"/>
+      <c r="C5" s="12">
+        <v>5</v>
+      </c>
+      <c r="D5" s="10"/>
+      <c r="E5" s="12">
+        <v>25</v>
+      </c>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="H5" s="13">
+        <f>_xlfn.PERCENTILE.INC(E2:E42,0.25)</f>
+        <v>40</v>
+      </c>
+      <c r="I5" s="10"/>
+      <c r="J5" s="10"/>
+    </row>
+    <row r="6" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A6" s="12">
+        <v>9</v>
+      </c>
+      <c r="B6" s="10"/>
+      <c r="C6" s="12">
+        <v>5</v>
+      </c>
+      <c r="D6" s="10"/>
+      <c r="E6" s="12">
+        <v>30</v>
+      </c>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="H6" s="13">
+        <f>MEDIAN(E2:E42)</f>
+        <v>50</v>
+      </c>
+      <c r="I6" s="10"/>
+      <c r="J6" s="10"/>
+    </row>
+    <row r="7" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A7" s="12">
+        <v>10</v>
+      </c>
+      <c r="B7" s="10"/>
+      <c r="C7" s="12">
+        <v>6</v>
+      </c>
+      <c r="D7" s="10"/>
+      <c r="E7" s="12">
+        <v>32</v>
+      </c>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="H7" s="13">
+        <f>_xlfn.PERCENTILE.INC(E2:E42,0.75)</f>
+        <v>60</v>
+      </c>
+      <c r="I7" s="10"/>
+      <c r="J7" s="10"/>
+    </row>
+    <row r="8" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A8" s="12">
+        <v>12</v>
+      </c>
+      <c r="B8" s="10"/>
+      <c r="C8" s="12">
+        <v>7</v>
+      </c>
+      <c r="D8" s="10"/>
+      <c r="E8" s="12">
+        <v>34</v>
+      </c>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="H8" s="13">
+        <f>H7-H5</f>
+        <v>20</v>
+      </c>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
+    </row>
+    <row r="9" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A9" s="12">
+        <v>13</v>
+      </c>
+      <c r="B9" s="10"/>
+      <c r="C9" s="12">
+        <v>8</v>
+      </c>
+      <c r="D9" s="10"/>
+      <c r="E9" s="12">
+        <v>36</v>
+      </c>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10"/>
+    </row>
+    <row r="10" spans="1:10" ht="36" customHeight="1">
+      <c r="A10" s="12">
+        <v>15</v>
+      </c>
+      <c r="B10" s="10"/>
+      <c r="C10" s="12">
+        <v>9</v>
+      </c>
+      <c r="D10" s="10"/>
+      <c r="E10" s="12">
+        <v>38</v>
+      </c>
+      <c r="F10" s="10"/>
+      <c r="G10" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="H10" s="17"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10"/>
+    </row>
+    <row r="11" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A11" s="12">
+        <v>18</v>
+      </c>
+      <c r="B11" s="10"/>
+      <c r="C11" s="12">
+        <v>31</v>
+      </c>
+      <c r="D11" s="10"/>
+      <c r="E11" s="12">
+        <v>40</v>
+      </c>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="10"/>
+    </row>
+    <row r="12" spans="1:10" ht="36" customHeight="1">
+      <c r="A12" s="12">
+        <v>22</v>
+      </c>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="12">
+        <v>40</v>
+      </c>
+      <c r="F12" s="10"/>
+      <c r="G12" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="H12" s="17"/>
+      <c r="I12" s="10"/>
+      <c r="J12" s="10"/>
+    </row>
+    <row r="13" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A13" s="10"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="12">
+        <v>42</v>
+      </c>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10"/>
+      <c r="J13" s="10"/>
+    </row>
+    <row r="14" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A14" s="10"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="12">
+        <v>44</v>
+      </c>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="10"/>
+      <c r="J14" s="10"/>
+    </row>
+    <row r="15" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A15" s="10"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="12">
+        <v>44</v>
+      </c>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+    </row>
+    <row r="16" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A16" s="10"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="12">
+        <v>46</v>
+      </c>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="10"/>
+      <c r="J16" s="10"/>
+    </row>
+    <row r="17" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A17" s="10"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="12">
+        <v>46</v>
+      </c>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="10"/>
+      <c r="J17" s="10"/>
+    </row>
+    <row r="18" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A18" s="10"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="12">
+        <v>48</v>
+      </c>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+    </row>
+    <row r="19" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A19" s="10"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="12">
+        <v>48</v>
+      </c>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+    </row>
+    <row r="20" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A20" s="10"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="12">
+        <v>49</v>
+      </c>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="10"/>
+      <c r="J20" s="10"/>
+    </row>
+    <row r="21" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A21" s="10"/>
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="12">
+        <v>50</v>
+      </c>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="10"/>
+      <c r="J21" s="10"/>
+    </row>
+    <row r="22" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A22" s="10"/>
+      <c r="B22" s="10"/>
+      <c r="C22" s="10"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="12">
+        <v>50</v>
+      </c>
+      <c r="F22" s="10"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="10"/>
+      <c r="I22" s="10"/>
+      <c r="J22" s="10"/>
+    </row>
+    <row r="23" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A23" s="10"/>
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="12">
+        <v>50</v>
+      </c>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
+    </row>
+    <row r="24" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A24" s="10"/>
+      <c r="B24" s="10"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="12">
+        <v>51</v>
+      </c>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="10"/>
+      <c r="I24" s="10"/>
+      <c r="J24" s="10"/>
+    </row>
+    <row r="25" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A25" s="10"/>
+      <c r="B25" s="10"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="12">
+        <v>52</v>
+      </c>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="10"/>
+      <c r="I25" s="10"/>
+      <c r="J25" s="10"/>
+    </row>
+    <row r="26" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A26" s="10"/>
+      <c r="B26" s="10"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="12">
+        <v>52</v>
+      </c>
+      <c r="F26" s="10"/>
+      <c r="G26" s="10"/>
+      <c r="H26" s="10"/>
+      <c r="I26" s="10"/>
+      <c r="J26" s="10"/>
+    </row>
+    <row r="27" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A27" s="10"/>
+      <c r="B27" s="10"/>
+      <c r="C27" s="10"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="12">
+        <v>54</v>
+      </c>
+      <c r="F27" s="10"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="10"/>
+      <c r="J27" s="10"/>
+    </row>
+    <row r="28" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A28" s="10"/>
+      <c r="B28" s="10"/>
+      <c r="C28" s="10"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="12">
+        <v>54</v>
+      </c>
+      <c r="F28" s="10"/>
+      <c r="G28" s="10"/>
+      <c r="H28" s="10"/>
+      <c r="I28" s="10"/>
+      <c r="J28" s="10"/>
+    </row>
+    <row r="29" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A29" s="10"/>
+      <c r="B29" s="10"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="12">
+        <v>56</v>
+      </c>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+    </row>
+    <row r="30" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A30" s="10"/>
+      <c r="B30" s="10"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="12">
+        <v>56</v>
+      </c>
+      <c r="F30" s="10"/>
+      <c r="G30" s="10"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="10"/>
+      <c r="J30" s="10"/>
+    </row>
+    <row r="31" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A31" s="10"/>
+      <c r="B31" s="10"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="12">
+        <v>58</v>
+      </c>
+      <c r="F31" s="10"/>
+      <c r="G31" s="10"/>
+      <c r="H31" s="10"/>
+      <c r="I31" s="10"/>
+      <c r="J31" s="10"/>
+    </row>
+    <row r="32" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A32" s="10"/>
+      <c r="B32" s="10"/>
+      <c r="C32" s="10"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="12">
+        <v>60</v>
+      </c>
+      <c r="F32" s="10"/>
+      <c r="G32" s="10"/>
+      <c r="H32" s="10"/>
+      <c r="I32" s="10"/>
+      <c r="J32" s="10"/>
+    </row>
+    <row r="33" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A33" s="10"/>
+      <c r="B33" s="10"/>
+      <c r="C33" s="10"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="12">
+        <v>60</v>
+      </c>
+      <c r="F33" s="10"/>
+      <c r="G33" s="10"/>
+      <c r="H33" s="10"/>
+      <c r="I33" s="10"/>
+      <c r="J33" s="10"/>
+    </row>
+    <row r="34" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A34" s="10"/>
+      <c r="B34" s="10"/>
+      <c r="C34" s="10"/>
+      <c r="D34" s="10"/>
+      <c r="E34" s="12">
+        <v>62</v>
+      </c>
+      <c r="F34" s="10"/>
+      <c r="G34" s="10"/>
+      <c r="H34" s="10"/>
+      <c r="I34" s="10"/>
+      <c r="J34" s="10"/>
+    </row>
+    <row r="35" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A35" s="10"/>
+      <c r="B35" s="10"/>
+      <c r="C35" s="10"/>
+      <c r="D35" s="10"/>
+      <c r="E35" s="12">
+        <v>64</v>
+      </c>
+      <c r="F35" s="10"/>
+      <c r="G35" s="10"/>
+      <c r="H35" s="10"/>
+      <c r="I35" s="10"/>
+      <c r="J35" s="10"/>
+    </row>
+    <row r="36" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A36" s="10"/>
+      <c r="B36" s="10"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="10"/>
+      <c r="E36" s="12">
+        <v>66</v>
+      </c>
+      <c r="F36" s="10"/>
+      <c r="G36" s="10"/>
+      <c r="H36" s="10"/>
+      <c r="I36" s="10"/>
+      <c r="J36" s="10"/>
+    </row>
+    <row r="37" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A37" s="10"/>
+      <c r="B37" s="10"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="10"/>
+      <c r="E37" s="12">
+        <v>68</v>
+      </c>
+      <c r="F37" s="10"/>
+      <c r="G37" s="10"/>
+      <c r="H37" s="10"/>
+      <c r="I37" s="10"/>
+      <c r="J37" s="10"/>
+    </row>
+    <row r="38" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A38" s="10"/>
+      <c r="B38" s="10"/>
+      <c r="C38" s="10"/>
+      <c r="D38" s="10"/>
+      <c r="E38" s="12">
+        <v>70</v>
+      </c>
+      <c r="F38" s="10"/>
+      <c r="G38" s="10"/>
+      <c r="H38" s="10"/>
+      <c r="I38" s="10"/>
+      <c r="J38" s="10"/>
+    </row>
+    <row r="39" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A39" s="10"/>
+      <c r="B39" s="10"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="12">
+        <v>75</v>
+      </c>
+      <c r="F39" s="10"/>
+      <c r="G39" s="10"/>
+      <c r="H39" s="10"/>
+      <c r="I39" s="10"/>
+      <c r="J39" s="10"/>
+    </row>
+    <row r="40" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A40" s="10"/>
+      <c r="B40" s="10"/>
+      <c r="C40" s="10"/>
+      <c r="D40" s="10"/>
+      <c r="E40" s="12">
+        <v>85</v>
+      </c>
+      <c r="F40" s="10"/>
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="I40" s="10"/>
+      <c r="J40" s="10"/>
+    </row>
+    <row r="41" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A41" s="10"/>
+      <c r="B41" s="10"/>
+      <c r="C41" s="10"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="12">
+        <v>95</v>
+      </c>
+      <c r="F41" s="10"/>
+      <c r="G41" s="10"/>
+      <c r="H41" s="10"/>
+      <c r="I41" s="10"/>
+      <c r="J41" s="10"/>
+    </row>
+    <row r="42" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A42" s="10"/>
+      <c r="B42" s="10"/>
+      <c r="C42" s="10"/>
+      <c r="D42" s="10"/>
+      <c r="E42" s="12">
+        <v>98</v>
+      </c>
+      <c r="F42" s="10"/>
+      <c r="G42" s="10"/>
+      <c r="H42" s="10"/>
+      <c r="I42" s="10"/>
+      <c r="J42" s="10"/>
+    </row>
+    <row r="43" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A43" s="10"/>
+      <c r="B43" s="10"/>
+      <c r="C43" s="10"/>
+      <c r="D43" s="10"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="10"/>
+      <c r="I43" s="10"/>
+      <c r="J43" s="10"/>
+    </row>
+    <row r="44" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A44" s="10"/>
+      <c r="B44" s="10"/>
+      <c r="C44" s="10"/>
+      <c r="D44" s="10"/>
+      <c r="E44" s="10"/>
+      <c r="F44" s="10"/>
+      <c r="G44" s="10"/>
+      <c r="H44" s="10"/>
+      <c r="I44" s="10"/>
+      <c r="J44" s="10"/>
+    </row>
+    <row r="45" spans="1:10" ht="22.95" customHeight="1">
+      <c r="A45" s="10"/>
+      <c r="B45" s="10"/>
+      <c r="C45" s="10"/>
+      <c r="D45" s="10"/>
+      <c r="E45" s="10"/>
+      <c r="F45" s="10"/>
+      <c r="G45" s="10"/>
+      <c r="H45" s="10"/>
+      <c r="I45" s="10"/>
+      <c r="J45" s="10"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="G12:H12"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:J40"/>
   <sheetFormatPr defaultRowHeight="13.6"/>
@@ -2813,37 +3645,37 @@
   <sheetData>
     <row r="1" spans="1:10" ht="36" customHeight="1">
       <c r="A1" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F1" s="1"/>
+      <c r="G1" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F1" s="1"/>
-      <c r="G1" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="H1" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="I1" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="J1" s="11" t="s">
-        <v>79</v>
+      <c r="H1" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="I1" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="J1" s="14" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="22.95" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="B2" s="9">
         <v>6</v>
@@ -2852,7 +3684,7 @@
         <v>5</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E2" s="3">
         <v>2</v>
@@ -2865,7 +3697,7 @@
     </row>
     <row r="3" spans="1:10" ht="36" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="B3" s="9">
         <v>8</v>
@@ -2874,28 +3706,28 @@
         <v>9</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E3" s="3">
         <v>4</v>
       </c>
       <c r="F3" s="1"/>
-      <c r="G3" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="H3" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="I3" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="J3" s="11" t="s">
-        <v>84</v>
+      <c r="G3" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="H3" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="I3" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="J3" s="14" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="22.95" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="B4" s="9">
         <v>7</v>
@@ -2904,7 +3736,7 @@
         <v>8</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E4" s="3">
         <v>3</v>
@@ -2917,7 +3749,7 @@
     </row>
     <row r="5" spans="1:10" ht="36" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="B5" s="9">
         <v>5</v>
@@ -2926,35 +3758,35 @@
         <v>6</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E5" s="3">
         <v>2</v>
       </c>
       <c r="F5" s="1"/>
-      <c r="G5" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="H5" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="I5" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="J5" s="11" t="s">
-        <v>87</v>
+      <c r="G5" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="H5" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="I5" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="J5" s="14" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="22.95" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B6" s="9"/>
       <c r="C6" s="3">
         <v>7</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E6" s="3">
         <v>3</v>
@@ -2967,7 +3799,7 @@
     </row>
     <row r="7" spans="1:10" ht="36" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="B7" s="9">
         <v>7</v>
@@ -2976,28 +3808,28 @@
         <v>0</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E7" s="3">
         <v>1</v>
       </c>
       <c r="F7" s="1"/>
-      <c r="G7" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="I7" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="J7" s="11" t="s">
-        <v>90</v>
+      <c r="G7" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="H7" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="I7" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="J7" s="14" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="22.95" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="B8" s="9">
         <v>4.5</v>
@@ -3006,7 +3838,7 @@
         <v>2</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E8" s="3">
         <v>1</v>
@@ -3019,7 +3851,7 @@
     </row>
     <row r="9" spans="1:10" ht="36" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B9" s="9">
         <v>6.3</v>
@@ -3028,28 +3860,28 @@
         <v>7</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E9" s="3">
         <v>3</v>
       </c>
       <c r="F9" s="1"/>
-      <c r="G9" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="H9" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="I9" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="J9" s="11" t="s">
-        <v>93</v>
+      <c r="G9" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="H9" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="I9" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="J9" s="14" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="22.95" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B10" s="9">
         <v>7.3</v>
@@ -3058,7 +3890,7 @@
         <v>9</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E10" s="3">
         <v>4</v>
@@ -3071,7 +3903,7 @@
     </row>
     <row r="11" spans="1:10" ht="36" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B11" s="9">
         <v>8.1</v>
@@ -3080,35 +3912,35 @@
         <v>4</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E11" s="3">
         <v>2</v>
       </c>
       <c r="F11" s="1"/>
-      <c r="G11" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="H11" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="I11" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="J11" s="11" t="s">
-        <v>96</v>
+      <c r="G11" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="H11" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="I11" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="J11" s="14" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="22.95" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="B12" s="9"/>
       <c r="C12" s="3">
         <v>7</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E12" s="3">
         <v>3</v>
@@ -3121,7 +3953,7 @@
     </row>
     <row r="13" spans="1:10" ht="36" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="B13" s="9">
         <v>6</v>
@@ -3130,28 +3962,28 @@
         <v>10</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E13" s="3">
         <v>2</v>
       </c>
       <c r="F13" s="1"/>
-      <c r="G13" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="H13" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="I13" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="J13" s="11" t="s">
-        <v>99</v>
+      <c r="G13" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="H13" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="I13" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="J13" s="14" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="22.95" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="B14" s="9">
         <v>7.1</v>
@@ -3160,7 +3992,7 @@
         <v>5</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E14" s="3">
         <v>3</v>
@@ -3173,7 +4005,7 @@
     </row>
     <row r="15" spans="1:10" ht="22.95" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B15" s="9">
         <v>7.9</v>
@@ -3182,7 +4014,7 @@
         <v>8</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E15" s="3">
         <v>1</v>
@@ -3195,7 +4027,7 @@
     </row>
     <row r="16" spans="1:10" ht="22.95" customHeight="1">
       <c r="A16" s="1" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="B16" s="9">
         <v>9.1999999999999993</v>
@@ -3204,7 +4036,7 @@
         <v>11</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E16" s="3">
         <v>3</v>
@@ -3217,7 +4049,7 @@
     </row>
     <row r="17" spans="1:10" ht="22.95" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="B17" s="9">
         <v>5.5</v>
@@ -3226,7 +4058,7 @@
         <v>6</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E17" s="3">
         <v>4</v>
@@ -3239,7 +4071,7 @@
     </row>
     <row r="18" spans="1:10" ht="22.95" customHeight="1">
       <c r="A18" s="1" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="B18" s="9">
         <v>6.8</v>
@@ -3248,7 +4080,7 @@
         <v>8</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E18" s="3">
         <v>2</v>
@@ -3261,7 +4093,7 @@
     </row>
     <row r="19" spans="1:10" ht="22.95" customHeight="1">
       <c r="A19" s="1" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="B19" s="9">
         <v>7.5</v>
@@ -3270,7 +4102,7 @@
         <v>3</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E19" s="3">
         <v>4</v>
@@ -3283,7 +4115,7 @@
     </row>
     <row r="20" spans="1:10" ht="22.95" customHeight="1">
       <c r="A20" s="1" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B20" s="9">
         <v>8.8000000000000007</v>
@@ -3292,7 +4124,7 @@
         <v>7</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E20" s="3">
         <v>2</v>
@@ -3305,7 +4137,7 @@
     </row>
     <row r="21" spans="1:10" ht="22.95" customHeight="1">
       <c r="A21" s="1" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B21" s="9">
         <v>4.8</v>
@@ -3314,7 +4146,7 @@
         <v>9</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E21" s="3">
         <v>3</v>
@@ -3327,7 +4159,7 @@
     </row>
     <row r="22" spans="1:10" ht="22.95" customHeight="1">
       <c r="A22" s="1" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B22" s="9">
         <v>6.5</v>
@@ -3336,7 +4168,7 @@
         <v>5</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E22" s="3">
         <v>1</v>
@@ -3349,7 +4181,7 @@
     </row>
     <row r="23" spans="1:10" ht="22.95" customHeight="1">
       <c r="A23" s="1" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B23" s="9">
         <v>7.4</v>
@@ -3358,7 +4190,7 @@
         <v>7</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E23" s="3">
         <v>3</v>
@@ -3371,7 +4203,7 @@
     </row>
     <row r="24" spans="1:10" ht="22.95" customHeight="1">
       <c r="A24" s="1" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B24" s="9">
         <v>8.3000000000000007</v>
@@ -3380,7 +4212,7 @@
         <v>10</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E24" s="3">
         <v>4</v>
@@ -3393,14 +4225,14 @@
     </row>
     <row r="25" spans="1:10" ht="22.95" customHeight="1">
       <c r="A25" s="1" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="B25" s="9"/>
       <c r="C25" s="3">
         <v>6</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E25" s="3">
         <v>3</v>
@@ -3413,7 +4245,7 @@
     </row>
     <row r="26" spans="1:10" ht="22.95" customHeight="1">
       <c r="A26" s="1" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="B26" s="9">
         <v>6.2</v>
@@ -3422,7 +4254,7 @@
         <v>8</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E26" s="3">
         <v>4</v>
@@ -3435,7 +4267,7 @@
     </row>
     <row r="27" spans="1:10" ht="22.95" customHeight="1">
       <c r="A27" s="1" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B27" s="9">
         <v>7.2</v>
@@ -3444,7 +4276,7 @@
         <v>12</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E27" s="3">
         <v>2</v>
@@ -3457,7 +4289,7 @@
     </row>
     <row r="28" spans="1:10" ht="22.95" customHeight="1">
       <c r="A28" s="1" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="B28" s="9">
         <v>8</v>
@@ -3466,7 +4298,7 @@
         <v>6</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E28" s="3">
         <v>3</v>
@@ -3479,7 +4311,7 @@
     </row>
     <row r="29" spans="1:10" ht="22.95" customHeight="1">
       <c r="A29" s="1" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B29" s="9">
         <v>9.5</v>
@@ -3488,7 +4320,7 @@
         <v>9</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E29" s="3">
         <v>2</v>
@@ -3501,7 +4333,7 @@
     </row>
     <row r="30" spans="1:10" ht="22.95" customHeight="1">
       <c r="A30" s="1" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="B30" s="9">
         <v>5.8</v>
@@ -3510,7 +4342,7 @@
         <v>4</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E30" s="3">
         <v>3</v>
@@ -3523,7 +4355,7 @@
     </row>
     <row r="31" spans="1:10" ht="22.95" customHeight="1">
       <c r="A31" s="1" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B31" s="9">
         <v>7</v>
@@ -3532,7 +4364,7 @@
         <v>7</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E31" s="3">
         <v>4</v>
@@ -3545,7 +4377,7 @@
     </row>
     <row r="32" spans="1:10" ht="22.95" customHeight="1">
       <c r="A32" s="1" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="B32" s="9">
         <v>7.7</v>
@@ -3554,7 +4386,7 @@
         <v>10</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E32" s="3">
         <v>3</v>
@@ -3567,7 +4399,7 @@
     </row>
     <row r="33" spans="1:10" ht="22.95" customHeight="1">
       <c r="A33" s="1" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="B33" s="9">
         <v>9</v>
@@ -3576,7 +4408,7 @@
         <v>5</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E33" s="3">
         <v>4</v>
@@ -3589,7 +4421,7 @@
     </row>
     <row r="34" spans="1:10" ht="22.95" customHeight="1">
       <c r="A34" s="1" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B34" s="9">
         <v>5.2</v>
@@ -3598,7 +4430,7 @@
         <v>8</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E34" s="3">
         <v>2</v>
@@ -3611,7 +4443,7 @@
     </row>
     <row r="35" spans="1:10" ht="22.95" customHeight="1">
       <c r="A35" s="1" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B35" s="9">
         <v>6.5</v>
@@ -3620,7 +4452,7 @@
         <v>11</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E35" s="3">
         <v>3</v>
@@ -3633,7 +4465,7 @@
     </row>
     <row r="36" spans="1:10" ht="22.95" customHeight="1">
       <c r="A36" s="1" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B36" s="9">
         <v>7.5</v>
@@ -3642,7 +4474,7 @@
         <v>6</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E36" s="3">
         <v>2</v>
@@ -3655,7 +4487,7 @@
     </row>
     <row r="37" spans="1:10" ht="22.95" customHeight="1">
       <c r="A37" s="1" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B37" s="9">
         <v>8.5</v>
@@ -3664,7 +4496,7 @@
         <v>8</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E37" s="3">
         <v>3</v>

</xml_diff>

<commit_message>
Revise chapter 3: remove repetition, add centre exceptions, introduce μ and σ²
- Czech labels in figure 3.3 (adapted, CC BY-SA 3.0)
- New figure with two discrete counterexamples to the mean/median/mode
  ordering after von Hippel (2005); frequencies in workbook sheet Vyjimky_stredu
- Trim repeated caveats; present linear interpolation as the textbook rule
  computed by PERCENTIL.INC (refinement of R04)
- Explain range growth, winsorizing replacements, whisker lengths, b = 0,
  and why the n vs n-1 bias matters for small n
- Introduce population μ, σ² and σ in chapter 3 (R36); chapter 4 recalls them
- Restore table attributes and blank lines lost in the author's edits
- Extend chapter 3 R checks; update maps, decisions and history

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kapitola_03.xlsx
+++ b/data/kapitola_03.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B276FE4-BA30-4E36-BEDB-2BFDD9A56E07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CCAB1DDE-4260-4091-8E13-11EBE6B2FB67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-109" yWindow="-109" windowWidth="34995" windowHeight="19060" xr2:uid="{A8ADB0FD-51A6-434D-B92F-D0A8272CE106}"/>
+    <workbookView xWindow="-109" yWindow="-109" windowWidth="34995" windowHeight="19060" xr2:uid="{D7D29B68-A21C-4A1C-9ED6-C1B3982A3EA6}"/>
   </bookViews>
   <sheets>
     <sheet name="Prehled" sheetId="1" r:id="rId1"/>
@@ -22,23 +22,24 @@
     <sheet name="Transformace" sheetId="12" r:id="rId12"/>
     <sheet name="Ordinalni_kvantily" sheetId="13" r:id="rId13"/>
     <sheet name="Vazeny_prumer" sheetId="14" r:id="rId14"/>
-    <sheet name="Kvantily" sheetId="15" r:id="rId15"/>
-    <sheet name="Orezani" sheetId="16" r:id="rId16"/>
-    <sheet name="Boxplot" sheetId="17" r:id="rId17"/>
-    <sheet name="Populace" sheetId="18" r:id="rId18"/>
-    <sheet name="Spicatost" sheetId="19" r:id="rId19"/>
-    <sheet name="U01_stred" sheetId="20" r:id="rId20"/>
-    <sheet name="U02_skupiny" sheetId="21" r:id="rId21"/>
-    <sheet name="U03_kvantily" sheetId="22" r:id="rId22"/>
-    <sheet name="U04_kategorie" sheetId="23" r:id="rId23"/>
-    <sheet name="U05_variabilita" sheetId="24" r:id="rId24"/>
-    <sheet name="U06_simulace" sheetId="25" r:id="rId25"/>
-    <sheet name="U07_MedAD" sheetId="26" r:id="rId26"/>
-    <sheet name="U09_boxplot" sheetId="27" r:id="rId27"/>
-    <sheet name="U10_transformace" sheetId="28" r:id="rId28"/>
-    <sheet name="U11_strategie" sheetId="29" r:id="rId29"/>
-    <sheet name="Entropie_data" sheetId="30" r:id="rId30"/>
-    <sheet name="U14_sikmost" sheetId="31" r:id="rId31"/>
+    <sheet name="Vyjimky_stredu" sheetId="15" r:id="rId15"/>
+    <sheet name="Kvantily" sheetId="16" r:id="rId16"/>
+    <sheet name="Orezani" sheetId="17" r:id="rId17"/>
+    <sheet name="Boxplot" sheetId="18" r:id="rId18"/>
+    <sheet name="Populace" sheetId="19" r:id="rId19"/>
+    <sheet name="Spicatost" sheetId="20" r:id="rId20"/>
+    <sheet name="U01_stred" sheetId="21" r:id="rId21"/>
+    <sheet name="U02_skupiny" sheetId="22" r:id="rId22"/>
+    <sheet name="U03_kvantily" sheetId="23" r:id="rId23"/>
+    <sheet name="U04_kategorie" sheetId="24" r:id="rId24"/>
+    <sheet name="U05_variabilita" sheetId="25" r:id="rId25"/>
+    <sheet name="U06_simulace" sheetId="26" r:id="rId26"/>
+    <sheet name="U07_MedAD" sheetId="27" r:id="rId27"/>
+    <sheet name="U09_boxplot" sheetId="28" r:id="rId28"/>
+    <sheet name="U10_transformace" sheetId="29" r:id="rId29"/>
+    <sheet name="U11_strategie" sheetId="30" r:id="rId30"/>
+    <sheet name="Entropie_data" sheetId="31" r:id="rId31"/>
+    <sheet name="U14_sikmost" sheetId="32" r:id="rId32"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -64,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="279">
   <si>
     <t>Doba (min)</t>
   </si>
@@ -372,6 +373,24 @@
     <t>Zadány jsou pouze velikosti skupin a průměry. Jednotlivé časy nejsou známy.</t>
   </si>
   <si>
+    <t>Počet pokusů (A)</t>
+  </si>
+  <si>
+    <t>Četnost A</t>
+  </si>
+  <si>
+    <t>Počet chyb (B)</t>
+  </si>
+  <si>
+    <t>Četnost B</t>
+  </si>
+  <si>
+    <t>Obrázek: výjimky z pořadí ukazatelů středu</t>
+  </si>
+  <si>
+    <t>Autorské modelové četnosti: A 100 lidí, B 20 lidí. Řádek je hodnota s četností, nikoli jeden účastník.</t>
+  </si>
+  <si>
     <t>Výklad interpolace; cvičení 3 (druhá část)</t>
   </si>
   <si>
@@ -568,6 +587,12 @@
   </si>
   <si>
     <t>A2:C3</t>
+  </si>
+  <si>
+    <t>Vyjimky_stredu</t>
+  </si>
+  <si>
+    <t>A2:D6</t>
   </si>
   <si>
     <t>Kvantily</t>
@@ -1367,8 +1392,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4C8A02F-9191-4C00-9FDC-D621D5B1EE6D}">
-  <dimension ref="A1:C40"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A36091D-B699-4AAA-AF0E-9E2E085BB8A2}">
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="25.625" customWidth="1"/>
@@ -1377,7 +1402,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -1389,49 +1414,49 @@
     </row>
     <row r="3" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="B3" s="11"/>
       <c r="C3" s="11"/>
     </row>
     <row r="4" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="B4" s="11"/>
       <c r="C4" s="11"/>
     </row>
     <row r="5" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="11"/>
     </row>
     <row r="6" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
     </row>
     <row r="7" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>75</v>
@@ -1439,10 +1464,10 @@
     </row>
     <row r="9" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>79</v>
@@ -1450,10 +1475,10 @@
     </row>
     <row r="10" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>82</v>
@@ -1461,10 +1486,10 @@
     </row>
     <row r="11" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>83</v>
@@ -1472,10 +1497,10 @@
     </row>
     <row r="12" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>84</v>
@@ -1483,10 +1508,10 @@
     </row>
     <row r="13" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>86</v>
@@ -1494,10 +1519,10 @@
     </row>
     <row r="14" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>95</v>
@@ -1505,10 +1530,10 @@
     </row>
     <row r="15" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>100</v>
@@ -1516,153 +1541,153 @@
     </row>
     <row r="16" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>156</v>
+        <v>181</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>176</v>
+        <v>162</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>167</v>
+        <v>186</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>156</v>
+        <v>194</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>189</v>
+        <v>162</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>176</v>
+        <v>197</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>139</v>
@@ -1670,96 +1695,102 @@
     </row>
     <row r="30" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>196</v>
+        <v>152</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="1"/>
-      <c r="B38" s="1"/>
-      <c r="C38" s="1"/>
+      <c r="A38" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>216</v>
+      </c>
     </row>
     <row r="39" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
@@ -1770,6 +1801,11 @@
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
+    </row>
+    <row r="41" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="1"/>
+      <c r="B41" s="1"/>
+      <c r="C41" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1784,7 +1820,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E861FB51-F94A-4323-9101-84308C9CFE72}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BA66BDA-5A2E-4270-B53F-4CB20F9C772C}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1844,7 +1880,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6825C2DE-0044-4B42-836E-F9055BE64E16}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B8A66B6-E157-4922-BD8A-825415555063}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1904,7 +1940,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF12CB68-1C0E-475A-A617-036F089251C8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{828EC7BA-5756-4CE1-AFE0-10147960868A}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1964,7 +2000,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37DEB4DA-8E0A-43C6-9646-E3ACEAB565BF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22BE8489-7A46-4CDE-9B71-E92697C47435}">
   <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2069,7 +2105,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D0AF713-6DF1-4B88-AC25-F23A9E36FD55}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FDA6D2E-2723-4A90-81D1-11427B0A3BD0}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2141,7 +2177,124 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75A6BF2A-1F5D-4991-A5A2-0CEE41D1C772}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD039765-5C9E-4499-9BF7-20A77D8B8B91}">
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="4" width="22.625" customWidth="1"/>
+    <col min="6" max="6" width="60.625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="F1" s="17" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="16">
+        <v>1</v>
+      </c>
+      <c r="B2" s="16">
+        <v>38</v>
+      </c>
+      <c r="C2" s="16">
+        <v>0</v>
+      </c>
+      <c r="D2" s="16">
+        <v>8</v>
+      </c>
+      <c r="F2" s="19" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="16">
+        <v>2</v>
+      </c>
+      <c r="B3" s="16">
+        <v>49</v>
+      </c>
+      <c r="C3" s="16">
+        <v>1</v>
+      </c>
+      <c r="D3" s="16">
+        <v>7</v>
+      </c>
+      <c r="F3" s="18"/>
+    </row>
+    <row r="4" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="16">
+        <v>3</v>
+      </c>
+      <c r="B4" s="16">
+        <v>8</v>
+      </c>
+      <c r="C4" s="16">
+        <v>2</v>
+      </c>
+      <c r="D4" s="16">
+        <v>3</v>
+      </c>
+      <c r="F4" s="19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="16">
+        <v>4</v>
+      </c>
+      <c r="B5" s="16">
+        <v>3</v>
+      </c>
+      <c r="C5" s="16">
+        <v>3</v>
+      </c>
+      <c r="D5" s="16">
+        <v>1</v>
+      </c>
+      <c r="F5" s="18"/>
+    </row>
+    <row r="6" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="16">
+        <v>5</v>
+      </c>
+      <c r="B6" s="16">
+        <v>2</v>
+      </c>
+      <c r="C6" s="16">
+        <v>4</v>
+      </c>
+      <c r="D6" s="16">
+        <v>1</v>
+      </c>
+      <c r="F6" s="18"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F7" s="18"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="F4:F7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15CC0FEC-3F3F-4D5A-AACF-0CF716293F97}">
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2162,7 +2315,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2231,8 +2384,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8B41C27-9AC4-4855-8BDE-7DFD321AA395}">
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72383AAC-BB00-4E1E-BDCE-2FB075C99471}">
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2253,7 +2406,7 @@
         <v>2</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2306,247 +2459,6 @@
     <row r="11" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="16">
         <v>31</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="C4:C7"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A542DCDB-0D9B-488A-83D3-9FAEBC91A248}">
-  <dimension ref="A1:C42"/>
-  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="22.625" customWidth="1"/>
-    <col min="3" max="3" width="60.625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="C1" s="17" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16">
-        <v>2</v>
-      </c>
-      <c r="C2" s="19" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="16">
-        <v>5</v>
-      </c>
-      <c r="C3" s="18"/>
-    </row>
-    <row r="4" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="16">
-        <v>15</v>
-      </c>
-      <c r="C4" s="19" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="16">
-        <v>25</v>
-      </c>
-      <c r="C5" s="18"/>
-    </row>
-    <row r="6" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="16">
-        <v>30</v>
-      </c>
-      <c r="C6" s="18"/>
-    </row>
-    <row r="7" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="16">
-        <v>32</v>
-      </c>
-      <c r="C7" s="18"/>
-    </row>
-    <row r="8" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="16">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="16">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="16">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="16">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="16">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="16">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="16">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="16">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="16">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="16">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="16">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="16">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="16">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="16">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="16">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="16">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="16">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="16">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="16">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="16">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="16">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="16">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="16">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="16">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="16">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="16">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="16">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="16">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="16">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="16">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="16">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="16">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="16">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="41" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="16">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="16">
-        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -2559,7 +2471,248 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB6E858E-C2F8-4BA5-A51D-E335EC6A8F04}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68B2B116-D191-423F-B656-1538A96494F3}">
+  <dimension ref="A1:C42"/>
+  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.625" customWidth="1"/>
+    <col min="3" max="3" width="60.625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C1" s="17" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="16">
+        <v>2</v>
+      </c>
+      <c r="C2" s="19" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="16">
+        <v>5</v>
+      </c>
+      <c r="C3" s="18"/>
+    </row>
+    <row r="4" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="16">
+        <v>15</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="16">
+        <v>25</v>
+      </c>
+      <c r="C5" s="18"/>
+    </row>
+    <row r="6" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="16">
+        <v>30</v>
+      </c>
+      <c r="C6" s="18"/>
+    </row>
+    <row r="7" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="16">
+        <v>32</v>
+      </c>
+      <c r="C7" s="18"/>
+    </row>
+    <row r="8" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="16">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="16">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="16">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="16">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="16">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="16">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="16">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="16">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="16">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="16">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="16">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="16">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="16">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="16">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="16">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="16">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="16">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="16">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="16">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="16">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="16">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="16">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="16">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="16">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="16">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="16">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="16">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="16">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="16">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="16">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="16">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="16">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="16">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="16">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="16">
+        <v>98</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="C4:C7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FF97176-80E6-4C5E-B80D-BA8A0CA0622B}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2580,7 +2733,7 @@
         <v>2</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2594,7 +2747,7 @@
         <v>6</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2621,107 +2774,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B68EB109-6D2C-47BC-B592-232E88A73AA3}">
-  <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="3" width="22.625" customWidth="1"/>
-    <col min="5" max="5" width="60.625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="E1" s="17" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16">
-        <v>-3</v>
-      </c>
-      <c r="B2" s="16">
-        <v>0</v>
-      </c>
-      <c r="C2" s="16">
-        <v>1</v>
-      </c>
-      <c r="E2" s="19" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="16">
-        <v>-1</v>
-      </c>
-      <c r="B3" s="16">
-        <v>10</v>
-      </c>
-      <c r="C3" s="16">
-        <v>9</v>
-      </c>
-      <c r="E3" s="18"/>
-    </row>
-    <row r="4" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="16">
-        <v>0</v>
-      </c>
-      <c r="B4" s="16">
-        <v>80</v>
-      </c>
-      <c r="C4" s="16">
-        <v>80</v>
-      </c>
-      <c r="E4" s="19" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="16">
-        <v>1</v>
-      </c>
-      <c r="B5" s="16">
-        <v>10</v>
-      </c>
-      <c r="C5" s="16">
-        <v>9</v>
-      </c>
-      <c r="E5" s="18"/>
-    </row>
-    <row r="6" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="16">
-        <v>3</v>
-      </c>
-      <c r="B6" s="16">
-        <v>0</v>
-      </c>
-      <c r="C6" s="16">
-        <v>1</v>
-      </c>
-      <c r="E6" s="18"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E7" s="18"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="E4:E7"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3508C226-F3FB-424E-B0A1-A9237C9CF547}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B32CBB1-D387-4C71-B8D4-F8C3116E6BD0}">
   <dimension ref="A1:J40"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3435,7 +3489,106 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B217EFA-ADE8-496D-BC9D-99C1CA2F37A7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FC26A3B-DD76-4EB0-86AD-9ACBB56ED4B5}">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="3" width="22.625" customWidth="1"/>
+    <col min="5" max="5" width="60.625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="E1" s="17" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="16">
+        <v>-3</v>
+      </c>
+      <c r="B2" s="16">
+        <v>0</v>
+      </c>
+      <c r="C2" s="16">
+        <v>1</v>
+      </c>
+      <c r="E2" s="19" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="16">
+        <v>-1</v>
+      </c>
+      <c r="B3" s="16">
+        <v>10</v>
+      </c>
+      <c r="C3" s="16">
+        <v>9</v>
+      </c>
+      <c r="E3" s="18"/>
+    </row>
+    <row r="4" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="16">
+        <v>0</v>
+      </c>
+      <c r="B4" s="16">
+        <v>80</v>
+      </c>
+      <c r="C4" s="16">
+        <v>80</v>
+      </c>
+      <c r="E4" s="19" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="16">
+        <v>1</v>
+      </c>
+      <c r="B5" s="16">
+        <v>10</v>
+      </c>
+      <c r="C5" s="16">
+        <v>9</v>
+      </c>
+      <c r="E5" s="18"/>
+    </row>
+    <row r="6" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="16">
+        <v>3</v>
+      </c>
+      <c r="B6" s="16">
+        <v>0</v>
+      </c>
+      <c r="C6" s="16">
+        <v>1</v>
+      </c>
+      <c r="E6" s="18"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E7" s="18"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="E4:E7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE3816AB-3C6D-4A62-8326-A2E848B784B2}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3456,7 +3609,7 @@
         <v>3</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3500,8 +3653,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A00483D3-785A-4CD9-89F8-324BA81B4AB3}">
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95AF0BCE-30B3-4775-9E9B-9E16C5DB462A}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3517,7 +3670,7 @@
         <v>98</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="E1" s="17" t="s">
         <v>74</v>
@@ -3534,7 +3687,7 @@
         <v>6</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3551,7 +3704,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E4" s="19" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -3572,8 +3725,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A37AC09-78F6-4F24-8CE4-79E9DFD88C46}">
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A52892D-0D9C-4F20-ABBF-2A54962339B0}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3583,7 +3736,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C1" s="17" t="s">
         <v>74</v>
@@ -3594,7 +3747,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3638,8 +3791,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DEC5B43-AEFF-441C-B8A9-1A8C668A9276}">
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F8E092A-7691-4C83-BD6F-62856CBD8CB7}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3649,10 +3802,10 @@
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="D1" s="17" t="s">
         <v>74</v>
@@ -3666,7 +3819,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3713,8 +3866,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FABC7676-1B3E-4BB0-92CB-C90700BFD004}">
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3560EFD2-122C-46B8-8AA9-B8522145956B}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3735,7 +3888,7 @@
         <v>2</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3770,8 +3923,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AC3B1EC-3628-4FD3-B7B8-50B57316FCD8}">
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{667B843C-A028-43D6-96BC-421A3330317F}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3782,13 +3935,13 @@
   <sheetData>
     <row r="1" spans="1:5" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>81</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="E1" s="17" t="s">
         <v>74</v>
@@ -3796,53 +3949,53 @@
     </row>
     <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="B2" s="16">
         <v>8</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="16" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="B3" s="16">
         <v>5</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="E3" s="18"/>
     </row>
     <row r="4" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B4" s="16">
         <v>6.41</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="B5" s="16">
         <v>8.01</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="E5" s="18"/>
     </row>
@@ -3861,8 +4014,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A828E74-52B2-4F0B-876C-7E6876E8FBBB}">
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AAFC72E-208C-4191-A9E7-1DD30DF255EC}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3883,7 +4036,7 @@
         <v>2</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3897,7 +4050,7 @@
         <v>4</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3924,8 +4077,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{534800E3-3B8E-4D5D-8991-3D516597E435}">
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5099556-9DD5-42A4-BAC7-3F3BEF9B94FF}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3946,7 +4099,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4000,8 +4153,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BF002C4-9114-4FD8-BD2E-97F5DE0FB3F0}">
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDD5E56E-717F-4FF0-A350-460B27310CC8}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4011,13 +4164,13 @@
   <sheetData>
     <row r="1" spans="1:5" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>81</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="E1" s="17" t="s">
         <v>74</v>
@@ -4031,10 +4184,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4045,7 +4198,7 @@
         <v>1.5</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="E3" s="18"/>
     </row>
@@ -4057,124 +4210,34 @@
         <v>3.5</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B5" s="16">
         <v>2</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="E5" s="18"/>
     </row>
     <row r="6" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="B6" s="16">
         <v>60</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>138</v>
-      </c>
-      <c r="E6" s="18"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E7" s="18"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="E4:E7"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1614535E-9533-4295-9291-1EBB0F66B4FE}">
-  <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="3" width="22.625" customWidth="1"/>
-    <col min="5" max="5" width="60.625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="E1" s="17" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="B2" s="16">
-        <v>20</v>
-      </c>
-      <c r="C2" s="16">
-        <v>5</v>
-      </c>
-      <c r="E2" s="19" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="B3" s="16">
-        <v>0</v>
-      </c>
-      <c r="C3" s="16">
-        <v>5</v>
-      </c>
-      <c r="E3" s="18"/>
-    </row>
-    <row r="4" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
-        <v>62</v>
-      </c>
-      <c r="B4" s="16">
-        <v>0</v>
-      </c>
-      <c r="C4" s="16">
-        <v>5</v>
-      </c>
-      <c r="E4" s="19" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="B5" s="16">
-        <v>0</v>
-      </c>
-      <c r="C5" s="16">
-        <v>5</v>
-      </c>
-      <c r="E5" s="18"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <v>144</v>
+      </c>
       <c r="E6" s="18"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -4190,7 +4253,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE57FA1D-0EE8-4496-BB52-840D52D569BD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CCB1E7D-2CE1-4776-84A2-1329E8433A71}">
   <dimension ref="A1:J40"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4802,7 +4865,97 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C41BE38E-0AE2-46A0-A9F0-6E61319C058F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16E49ACD-75A1-4D59-962C-6188512FA258}">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="3" width="22.625" customWidth="1"/>
+    <col min="5" max="5" width="60.625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="E1" s="17" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2" s="16">
+        <v>20</v>
+      </c>
+      <c r="C2" s="16">
+        <v>5</v>
+      </c>
+      <c r="E2" s="19" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" s="16">
+        <v>0</v>
+      </c>
+      <c r="C3" s="16">
+        <v>5</v>
+      </c>
+      <c r="E3" s="18"/>
+    </row>
+    <row r="4" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" s="16">
+        <v>0</v>
+      </c>
+      <c r="C4" s="16">
+        <v>5</v>
+      </c>
+      <c r="E4" s="19" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5" s="16">
+        <v>0</v>
+      </c>
+      <c r="C5" s="16">
+        <v>5</v>
+      </c>
+      <c r="E5" s="18"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E6" s="18"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E7" s="18"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="E4:E7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A8B5A60-88DE-4388-9F60-9C1B6D94ACC6}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4829,7 +4982,7 @@
         <v>4</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4849,7 +5002,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4876,8 +5029,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3614B32-FD6B-479D-99BA-6992569651F5}">
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{252AC3CB-F2B0-42A6-9F5E-1AF0B499090D}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4887,7 +5040,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>57</v>
@@ -4904,7 +5057,7 @@
         <v>4</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4952,7 +5105,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{879358D1-D4C8-4488-96CC-CD6288B42983}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C183400A-0A99-4097-9646-65844BE42CE8}">
   <dimension ref="A1:J40"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5539,7 +5692,7 @@
     <mergeCell ref="A14:J14"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="whole" operator="greaterThanOrEqual" showInputMessage="1" sqref="B2:B5" xr:uid="{4285167A-FC59-4E28-97F1-A1B953C5C2B0}">
+    <dataValidation type="whole" operator="greaterThanOrEqual" showInputMessage="1" sqref="B2:B5" xr:uid="{898EAEC6-915C-443A-A0DE-6195A9490D58}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -5548,7 +5701,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23512365-E731-4F07-B14A-2C24C25E8A21}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{671192B0-BE21-46FA-85DF-D5FB6E645775}">
   <dimension ref="A1:J42"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5564,15 +5717,15 @@
   <sheetData>
     <row r="1" spans="1:10" ht="44" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="4" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="4" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="F1" s="1"/>
       <c r="G1" s="4" t="s">
@@ -5601,7 +5754,7 @@
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="2" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="H2" s="7">
         <f>_xlfn.PERCENTILE.INC(A2:A12,0.17)</f>
@@ -5627,7 +5780,7 @@
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="2" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="H3" s="7">
         <f>AVERAGE(C2:C11)</f>
@@ -5653,7 +5806,7 @@
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="2" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="H4" s="7">
         <f>MEDIAN(C2:C11)</f>
@@ -5679,7 +5832,7 @@
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="2" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="H5" s="7">
         <f>_xlfn.PERCENTILE.INC(E2:E42,0.25)</f>
@@ -5705,7 +5858,7 @@
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="2" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="H6" s="7">
         <f>MEDIAN(E2:E42)</f>
@@ -5731,7 +5884,7 @@
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="2" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="H7" s="7">
         <f>_xlfn.PERCENTILE.INC(E2:E42,0.75)</f>
@@ -5757,7 +5910,7 @@
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="2" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="H8" s="7">
         <f>H7-H5</f>
@@ -5804,7 +5957,7 @@
       </c>
       <c r="F10" s="1"/>
       <c r="G10" s="13" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="H10" s="14"/>
       <c r="I10" s="1"/>
@@ -5845,7 +5998,7 @@
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="13" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="H12" s="14"/>
       <c r="I12" s="1"/>
@@ -6293,7 +6446,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17775FA1-272A-4E6C-8B79-99FD63D4E644}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F45CC14-CC14-4049-8FD3-8CE5B28489CD}">
   <dimension ref="A1:J40"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -6304,23 +6457,23 @@
   <sheetData>
     <row r="1" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="F1" s="1"/>
       <c r="G1" s="13" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
@@ -6328,7 +6481,7 @@
     </row>
     <row r="2" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="B2" s="23">
         <v>6</v>
@@ -6337,7 +6490,7 @@
         <v>5</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E2" s="5">
         <v>2</v>
@@ -6350,7 +6503,7 @@
     </row>
     <row r="3" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="B3" s="23">
         <v>8</v>
@@ -6359,14 +6512,14 @@
         <v>9</v>
       </c>
       <c r="D3" s="20" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="E3" s="5">
         <v>4</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="13" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="H3" s="14"/>
       <c r="I3" s="14"/>
@@ -6374,7 +6527,7 @@
     </row>
     <row r="4" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="B4" s="23">
         <v>7</v>
@@ -6383,7 +6536,7 @@
         <v>8</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E4" s="5">
         <v>3</v>
@@ -6396,7 +6549,7 @@
     </row>
     <row r="5" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="B5" s="23">
         <v>5</v>
@@ -6405,14 +6558,14 @@
         <v>6</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="E5" s="5">
         <v>2</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="13" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
       <c r="H5" s="14"/>
       <c r="I5" s="14"/>
@@ -6420,14 +6573,14 @@
     </row>
     <row r="6" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="B6" s="23"/>
       <c r="C6" s="5">
         <v>7</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E6" s="5">
         <v>3</v>
@@ -6440,7 +6593,7 @@
     </row>
     <row r="7" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="B7" s="23">
         <v>7</v>
@@ -6449,14 +6602,14 @@
         <v>0</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="E7" s="5">
         <v>1</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="13" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="H7" s="14"/>
       <c r="I7" s="14"/>
@@ -6464,7 +6617,7 @@
     </row>
     <row r="8" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="B8" s="23">
         <v>4.5</v>
@@ -6473,7 +6626,7 @@
         <v>2</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="E8" s="5">
         <v>1</v>
@@ -6486,7 +6639,7 @@
     </row>
     <row r="9" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="B9" s="23">
         <v>6.3</v>
@@ -6495,14 +6648,14 @@
         <v>7</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E9" s="5">
         <v>3</v>
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="13" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
       <c r="H9" s="14"/>
       <c r="I9" s="14"/>
@@ -6510,7 +6663,7 @@
     </row>
     <row r="10" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="B10" s="23">
         <v>7.3</v>
@@ -6519,7 +6672,7 @@
         <v>9</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E10" s="5">
         <v>4</v>
@@ -6532,7 +6685,7 @@
     </row>
     <row r="11" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="B11" s="23">
         <v>8.1</v>
@@ -6541,14 +6694,14 @@
         <v>4</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="E11" s="5">
         <v>2</v>
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="13" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
       <c r="H11" s="14"/>
       <c r="I11" s="14"/>
@@ -6556,14 +6709,14 @@
     </row>
     <row r="12" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="B12" s="23"/>
       <c r="C12" s="5">
         <v>7</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E12" s="5">
         <v>3</v>
@@ -6576,7 +6729,7 @@
     </row>
     <row r="13" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="B13" s="23">
         <v>6</v>
@@ -6585,14 +6738,14 @@
         <v>10</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E13" s="5">
         <v>2</v>
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="13" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="H13" s="14"/>
       <c r="I13" s="14"/>
@@ -6600,7 +6753,7 @@
     </row>
     <row r="14" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="B14" s="23">
         <v>7.1</v>
@@ -6609,7 +6762,7 @@
         <v>5</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="E14" s="5">
         <v>3</v>
@@ -6622,7 +6775,7 @@
     </row>
     <row r="15" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="B15" s="23">
         <v>7.9</v>
@@ -6631,7 +6784,7 @@
         <v>8</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E15" s="5">
         <v>1</v>
@@ -6644,7 +6797,7 @@
     </row>
     <row r="16" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="B16" s="23">
         <v>9.1999999999999993</v>
@@ -6653,7 +6806,7 @@
         <v>11</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E16" s="5">
         <v>3</v>
@@ -6666,7 +6819,7 @@
     </row>
     <row r="17" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="B17" s="23">
         <v>5.5</v>
@@ -6675,7 +6828,7 @@
         <v>6</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="E17" s="5">
         <v>4</v>
@@ -6688,7 +6841,7 @@
     </row>
     <row r="18" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="B18" s="23">
         <v>6.8</v>
@@ -6697,7 +6850,7 @@
         <v>8</v>
       </c>
       <c r="D18" s="20" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E18" s="5">
         <v>2</v>
@@ -6710,7 +6863,7 @@
     </row>
     <row r="19" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="B19" s="23">
         <v>7.5</v>
@@ -6719,7 +6872,7 @@
         <v>3</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E19" s="5">
         <v>4</v>
@@ -6732,7 +6885,7 @@
     </row>
     <row r="20" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="B20" s="23">
         <v>8.8000000000000007</v>
@@ -6741,7 +6894,7 @@
         <v>7</v>
       </c>
       <c r="D20" s="20" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="E20" s="5">
         <v>2</v>
@@ -6754,7 +6907,7 @@
     </row>
     <row r="21" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="B21" s="23">
         <v>4.8</v>
@@ -6763,7 +6916,7 @@
         <v>9</v>
       </c>
       <c r="D21" s="20" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E21" s="5">
         <v>3</v>
@@ -6776,7 +6929,7 @@
     </row>
     <row r="22" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="B22" s="23">
         <v>6.5</v>
@@ -6785,7 +6938,7 @@
         <v>5</v>
       </c>
       <c r="D22" s="20" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E22" s="5">
         <v>1</v>
@@ -6798,7 +6951,7 @@
     </row>
     <row r="23" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="B23" s="23">
         <v>7.4</v>
@@ -6807,7 +6960,7 @@
         <v>7</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="E23" s="5">
         <v>3</v>
@@ -6820,7 +6973,7 @@
     </row>
     <row r="24" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="B24" s="23">
         <v>8.3000000000000007</v>
@@ -6829,7 +6982,7 @@
         <v>10</v>
       </c>
       <c r="D24" s="20" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E24" s="5">
         <v>4</v>
@@ -6842,14 +6995,14 @@
     </row>
     <row r="25" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="B25" s="23"/>
       <c r="C25" s="5">
         <v>6</v>
       </c>
       <c r="D25" s="20" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E25" s="5">
         <v>3</v>
@@ -6862,7 +7015,7 @@
     </row>
     <row r="26" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
       <c r="B26" s="23">
         <v>6.2</v>
@@ -6871,7 +7024,7 @@
         <v>8</v>
       </c>
       <c r="D26" s="20" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="E26" s="5">
         <v>4</v>
@@ -6884,7 +7037,7 @@
     </row>
     <row r="27" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="B27" s="23">
         <v>7.2</v>
@@ -6893,7 +7046,7 @@
         <v>12</v>
       </c>
       <c r="D27" s="20" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E27" s="5">
         <v>2</v>
@@ -6906,7 +7059,7 @@
     </row>
     <row r="28" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="B28" s="23">
         <v>8</v>
@@ -6915,7 +7068,7 @@
         <v>6</v>
       </c>
       <c r="D28" s="20" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E28" s="5">
         <v>3</v>
@@ -6928,7 +7081,7 @@
     </row>
     <row r="29" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="B29" s="23">
         <v>9.5</v>
@@ -6937,7 +7090,7 @@
         <v>9</v>
       </c>
       <c r="D29" s="20" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="E29" s="5">
         <v>2</v>
@@ -6950,7 +7103,7 @@
     </row>
     <row r="30" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="B30" s="23">
         <v>5.8</v>
@@ -6959,7 +7112,7 @@
         <v>4</v>
       </c>
       <c r="D30" s="20" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E30" s="5">
         <v>3</v>
@@ -6972,7 +7125,7 @@
     </row>
     <row r="31" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="B31" s="23">
         <v>7</v>
@@ -6981,7 +7134,7 @@
         <v>7</v>
       </c>
       <c r="D31" s="20" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E31" s="5">
         <v>4</v>
@@ -6994,7 +7147,7 @@
     </row>
     <row r="32" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="B32" s="23">
         <v>7.7</v>
@@ -7003,7 +7156,7 @@
         <v>10</v>
       </c>
       <c r="D32" s="20" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="E32" s="5">
         <v>3</v>
@@ -7016,7 +7169,7 @@
     </row>
     <row r="33" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="B33" s="23">
         <v>9</v>
@@ -7025,7 +7178,7 @@
         <v>5</v>
       </c>
       <c r="D33" s="20" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E33" s="5">
         <v>4</v>
@@ -7038,7 +7191,7 @@
     </row>
     <row r="34" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="B34" s="23">
         <v>5.2</v>
@@ -7047,7 +7200,7 @@
         <v>8</v>
       </c>
       <c r="D34" s="20" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E34" s="5">
         <v>2</v>
@@ -7060,7 +7213,7 @@
     </row>
     <row r="35" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="B35" s="23">
         <v>6.5</v>
@@ -7069,7 +7222,7 @@
         <v>11</v>
       </c>
       <c r="D35" s="20" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="E35" s="5">
         <v>3</v>
@@ -7082,7 +7235,7 @@
     </row>
     <row r="36" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="B36" s="23">
         <v>7.5</v>
@@ -7091,7 +7244,7 @@
         <v>6</v>
       </c>
       <c r="D36" s="20" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E36" s="5">
         <v>2</v>
@@ -7104,7 +7257,7 @@
     </row>
     <row r="37" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B37" s="23">
         <v>8.5</v>
@@ -7113,7 +7266,7 @@
         <v>8</v>
       </c>
       <c r="D37" s="20" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E37" s="5">
         <v>3</v>
@@ -7175,7 +7328,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0D202CC-284C-487E-990F-273AE9945C0A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1753A032-2588-4CA5-9429-EF10BD63D566}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -7238,7 +7391,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCD1218A-925B-4F18-AE1B-E046D8704F7C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7266524D-3FF4-4F6D-8E64-D2AB9AD15E47}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -7319,7 +7472,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07922FC4-5646-478B-84AB-BE4C5B9BC306}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82E5FF3B-C65D-4BCF-ADBF-75F2DD75DB91}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>

<commit_message>
Chapters 3-4: core shape indicators (skewness, excess) and Q-Q link
Chapter 3 gets a core section "Ukazatele tvaru" (R44): meaning of
skewness and excess kurtosis, a figure of models with zero/moderate/high
skewness and excess (tails highlighted), the equal-peak counterexample
and misconception warning moved out of the optional block, SKEW/KURT in
Excel and their limits. Formulas, moments and corrections stay optional.
New core exercise 13; optional exercises renumbered to 14-15.

Chapter 4 section on reading Q-Q deviations adds a table of SKEW/KURT
for the four simulations and explains the convergent information and
its limits; exercise 10 and the summary are extended.

Glossary, Excel overview, workbooks, checks and author docs updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kapitola_03.xlsx
+++ b/data/kapitola_03.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CCAB1DDE-4260-4091-8E13-11EBE6B2FB67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{07A78DEB-B80B-4C74-9752-CE08F813CBF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-109" yWindow="-109" windowWidth="34995" windowHeight="19060" xr2:uid="{D7D29B68-A21C-4A1C-9ED6-C1B3982A3EA6}"/>
+    <workbookView xWindow="-109" yWindow="-109" windowWidth="34995" windowHeight="19060" xr2:uid="{F9AAF36E-E5DB-4BD1-865C-AC2811E97730}"/>
   </bookViews>
   <sheets>
     <sheet name="Prehled" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
     <sheet name="U10_transformace" sheetId="29" r:id="rId29"/>
     <sheet name="U11_strategie" sheetId="30" r:id="rId30"/>
     <sheet name="Entropie_data" sheetId="31" r:id="rId31"/>
-    <sheet name="U14_sikmost" sheetId="32" r:id="rId32"/>
+    <sheet name="U15_sikmost" sheetId="32" r:id="rId32"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="283">
   <si>
     <t>Doba (min)</t>
   </si>
@@ -229,6 +229,18 @@
     <t>V původních jednotkách</t>
   </si>
   <si>
+    <t>Šikmost</t>
+  </si>
+  <si>
+    <t>Znaménko: delší chvost; bez jednotky</t>
+  </si>
+  <si>
+    <t>Exces</t>
+  </si>
+  <si>
+    <t>Kladný: více velmi vzdálených hodnot než u normálního modelu</t>
+  </si>
+  <si>
     <t>Spánek: tři údaje chybějí. Paměť: nula vybavených slov je platný výsledek.</t>
   </si>
   <si>
@@ -418,7 +430,7 @@
     <t>Četnost vpravo</t>
   </si>
   <si>
-    <t>Obrázek: stejný vrchol; cvičení 14</t>
+    <t>Obrázek: stejný vrchol; nepovinné cvičení 15</t>
   </si>
   <si>
     <t>Cvičení 1</t>
@@ -517,13 +529,13 @@
     <t>Cvičení 11</t>
   </si>
   <si>
-    <t>Výklad; nepovinné cvičení 13</t>
+    <t>Výklad; nepovinné cvičení 14</t>
   </si>
   <si>
     <t>Výchozí tři kategorie A–C; D je rozšíření s nulovou četností. Další varianta: 8, 0, 0, 0.</t>
   </si>
   <si>
-    <t>Nepovinné cvičení 14</t>
+    <t>Nepovinné cvičení 15</t>
   </si>
   <si>
     <t>Data ke kapitole 3</t>
@@ -670,7 +682,7 @@
     <t>Entropie_data</t>
   </si>
   <si>
-    <t>U14_sikmost</t>
+    <t>U15_sikmost</t>
   </si>
   <si>
     <t>Data</t>
@@ -1392,7 +1404,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A36091D-B699-4AAA-AF0E-9E2E085BB8A2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2654576-2F32-44D3-9017-22F06108880D}">
   <dimension ref="A1:C41"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1402,7 +1414,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -1414,382 +1426,382 @@
     </row>
     <row r="3" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B3" s="11"/>
       <c r="C3" s="11"/>
     </row>
     <row r="4" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="B4" s="11"/>
       <c r="C4" s="11"/>
     </row>
     <row r="5" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="11"/>
     </row>
     <row r="6" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
     </row>
     <row r="7" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="30.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -1820,7 +1832,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BA66BDA-5A2E-4270-B53F-4CB20F9C772C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B342932-2EB2-49BC-A346-6F4FB20FC651}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1833,7 +1845,7 @@
         <v>0</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1841,7 +1853,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1855,7 +1867,7 @@
         <v>6</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1880,7 +1892,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B8A66B6-E157-4922-BD8A-825415555063}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C0B7DF0-4A8A-4C9C-86F8-2A7A5A886086}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1890,10 +1902,10 @@
   <sheetData>
     <row r="1" spans="1:3" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1901,7 +1913,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1915,7 +1927,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1940,7 +1952,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{828EC7BA-5756-4CE1-AFE0-10147960868A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A13F61A-925E-476B-BBE4-5B7715108558}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1950,10 +1962,10 @@
   <sheetData>
     <row r="1" spans="1:3" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1961,7 +1973,7 @@
         <v>2</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1975,7 +1987,7 @@
         <v>8</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2000,7 +2012,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22BE8489-7A46-4CDE-9B71-E92697C47435}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6677D4BF-EA29-41FD-865F-76A1299890AD}">
   <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2010,24 +2022,24 @@
   <sheetData>
     <row r="1" spans="1:6" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="F1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B2" s="16">
         <v>1</v>
@@ -2039,12 +2051,12 @@
         <v>1</v>
       </c>
       <c r="F2" s="19" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="16" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B3" s="16">
         <v>2</v>
@@ -2059,7 +2071,7 @@
     </row>
     <row r="4" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B4" s="16">
         <v>2</v>
@@ -2071,12 +2083,12 @@
         <v>10</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B5" s="16">
         <v>1</v>
@@ -2105,7 +2117,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FDA6D2E-2723-4A90-81D1-11427B0A3BD0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{996DCEDF-C00A-4400-9AC7-F757020549FE}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2115,21 +2127,21 @@
   <sheetData>
     <row r="1" spans="1:5" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="E1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B2" s="16">
         <v>10</v>
@@ -2138,12 +2150,12 @@
         <v>4</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="16" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B3" s="16">
         <v>30</v>
@@ -2155,7 +2167,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E4" s="19" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -2177,7 +2189,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD039765-5C9E-4499-9BF7-20A77D8B8B91}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BA9B97D-265F-46C3-A005-C0429172C76A}">
   <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2187,19 +2199,19 @@
   <sheetData>
     <row r="1" spans="1:6" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="F1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2216,7 +2228,7 @@
         <v>8</v>
       </c>
       <c r="F2" s="19" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2248,7 +2260,7 @@
         <v>3</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2294,7 +2306,7 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15CC0FEC-3F3F-4D5A-AACF-0CF716293F97}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADF3A2AB-71A6-4687-A8F9-EEDCB09BE15A}">
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2307,7 +2319,7 @@
         <v>0</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2315,7 +2327,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2329,7 +2341,7 @@
         <v>7</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2385,7 +2397,7 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72383AAC-BB00-4E1E-BDCE-2FB075C99471}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80DF9EE1-72AA-46DA-AE8E-42BBD36930BD}">
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2398,7 +2410,7 @@
         <v>0</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2406,7 +2418,7 @@
         <v>2</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2420,7 +2432,7 @@
         <v>4</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2471,7 +2483,7 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68B2B116-D191-423F-B656-1538A96494F3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E8F53AC-962D-4DD2-9CE2-2D189AC6979C}">
   <dimension ref="A1:C42"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2481,10 +2493,10 @@
   <sheetData>
     <row r="1" spans="1:3" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2492,7 +2504,7 @@
         <v>2</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2506,7 +2518,7 @@
         <v>15</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2712,7 +2724,7 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FF97176-80E6-4C5E-B80D-BA8A0CA0622B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6966C14E-4D98-4ECF-A5E6-273012A39CE2}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2725,7 +2737,7 @@
         <v>0</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2733,7 +2745,7 @@
         <v>2</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2747,7 +2759,7 @@
         <v>6</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2775,7 +2787,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B32CBB1-D387-4C71-B8D4-F8C3116E6BD0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78BE72D9-8932-4247-B095-5ECD14A567FA}">
   <dimension ref="A1:J40"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3489,7 +3501,7 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FC26A3B-DD76-4EB0-86AD-9ACBB56ED4B5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A8E137F-CD24-4F21-B200-865581BFCDBA}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3499,16 +3511,16 @@
   <sheetData>
     <row r="1" spans="1:5" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="E1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3522,7 +3534,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3548,7 +3560,7 @@
         <v>80</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3588,7 +3600,7 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE3816AB-3C6D-4A62-8326-A2E848B784B2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62C37062-1EDC-4E12-A826-BF60CAA604D8}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3601,7 +3613,7 @@
         <v>0</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3609,7 +3621,7 @@
         <v>3</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3623,7 +3635,7 @@
         <v>4</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3654,7 +3666,7 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95AF0BCE-30B3-4775-9E9B-9E16C5DB462A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAB8B6BB-A270-4DD5-A7B3-4DA3A19F8C2F}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3664,21 +3676,21 @@
   <sheetData>
     <row r="1" spans="1:5" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="E1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B2" s="16">
         <v>8</v>
@@ -3687,12 +3699,12 @@
         <v>6</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="16" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B3" s="16">
         <v>12</v>
@@ -3704,7 +3716,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E4" s="19" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -3726,7 +3738,7 @@
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A52892D-0D9C-4F20-ABBF-2A54962339B0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10ADAF17-9EDE-4443-A515-7C5902184423}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3736,10 +3748,10 @@
   <sheetData>
     <row r="1" spans="1:3" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3747,7 +3759,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3761,7 +3773,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3792,7 +3804,7 @@
 </file>
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F8E092A-7691-4C83-BD6F-62856CBD8CB7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E669A4A-90F3-4E5F-9627-06A9E0C45848}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3802,29 +3814,29 @@
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="D1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B2" s="16">
         <v>1</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="16" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B3" s="16">
         <v>2</v>
@@ -3833,18 +3845,18 @@
     </row>
     <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B4" s="16">
         <v>3</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B5" s="16">
         <v>4</v>
@@ -3867,7 +3879,7 @@
 </file>
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3560EFD2-122C-46B8-8AA9-B8522145956B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87560C0C-DDD5-4FCA-A549-ADF405064AB5}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3880,7 +3892,7 @@
         <v>0</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3888,7 +3900,7 @@
         <v>2</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3902,7 +3914,7 @@
         <v>6</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -3924,7 +3936,7 @@
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{667B843C-A028-43D6-96BC-421A3330317F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{524ECB03-3DFD-4E8F-8D52-7E42EE8CD11C}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3935,67 +3947,67 @@
   <sheetData>
     <row r="1" spans="1:5" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="E1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B2" s="16">
         <v>8</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="16" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B3" s="16">
         <v>5</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="E3" s="18"/>
     </row>
     <row r="4" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B4" s="16">
         <v>6.41</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B5" s="16">
         <v>8.01</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="E5" s="18"/>
     </row>
@@ -4015,7 +4027,7 @@
 </file>
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AAFC72E-208C-4191-A9E7-1DD30DF255EC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EF1F987-4E28-4D9B-98F6-C3BF89C2FD09}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4028,7 +4040,7 @@
         <v>0</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4036,7 +4048,7 @@
         <v>2</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4050,7 +4062,7 @@
         <v>4</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4078,7 +4090,7 @@
 </file>
 
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5099556-9DD5-42A4-BAC7-3F3BEF9B94FF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73C5DBCB-FD1E-4CD0-93F3-32FF61BBBD85}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4091,7 +4103,7 @@
         <v>0</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4099,7 +4111,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4113,7 +4125,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4154,7 +4166,7 @@
 </file>
 
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDD5E56E-717F-4FF0-A350-460B27310CC8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4BBCF7B-1CE2-4E19-99FA-81DCB8D51643}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4164,16 +4176,16 @@
   <sheetData>
     <row r="1" spans="1:5" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="E1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4184,10 +4196,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4198,7 +4210,7 @@
         <v>1.5</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="E3" s="18"/>
     </row>
@@ -4210,33 +4222,33 @@
         <v>3.5</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B5" s="16">
         <v>2</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="E5" s="18"/>
     </row>
     <row r="6" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B6" s="16">
         <v>60</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="E6" s="18"/>
     </row>
@@ -4253,7 +4265,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CCB1E7D-2CE1-4776-84A2-1329E8433A71}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5B6C050-B2D2-4074-A4FA-801D1E85E9D9}">
   <dimension ref="A1:J40"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4504,10 +4516,20 @@
       <c r="J11" s="1"/>
     </row>
     <row r="12" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
+      <c r="A12" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" s="7">
+        <f>SKEW(Data!B2:B37)</f>
+        <v>-0.1250536524296447</v>
+      </c>
+      <c r="C12" s="7">
+        <f>SKEW(Data!C2:C37)</f>
+        <v>-0.47057774610161002</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>55</v>
+      </c>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
@@ -4516,10 +4538,20 @@
       <c r="J12" s="1"/>
     </row>
     <row r="13" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
+      <c r="A13" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" s="7">
+        <f>KURT(Data!B2:B37)</f>
+        <v>-0.55379448461620973</v>
+      </c>
+      <c r="C13" s="7">
+        <f>KURT(Data!C2:C37)</f>
+        <v>0.48140624763994788</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>57</v>
+      </c>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
@@ -4529,7 +4561,7 @@
     </row>
     <row r="14" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B14" s="14"/>
       <c r="C14" s="14"/>
@@ -4555,7 +4587,7 @@
     </row>
     <row r="16" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B16" s="14"/>
       <c r="C16" s="14"/>
@@ -4865,7 +4897,7 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16E49ACD-75A1-4D59-962C-6188512FA258}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4834D330-EE7C-4E24-9F14-8342558EA776}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4875,21 +4907,21 @@
   <sheetData>
     <row r="1" spans="1:5" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="E1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B2" s="16">
         <v>20</v>
@@ -4898,12 +4930,12 @@
         <v>5</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="16" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B3" s="16">
         <v>0</v>
@@ -4915,7 +4947,7 @@
     </row>
     <row r="4" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B4" s="16">
         <v>0</v>
@@ -4924,12 +4956,12 @@
         <v>5</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B5" s="16">
         <v>0</v>
@@ -4955,7 +4987,7 @@
 </file>
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A8B5A60-88DE-4388-9F60-9C1B6D94ACC6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB13C4D8-04A7-4D72-8B62-DB164218B5BA}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4965,29 +4997,29 @@
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B2" s="16">
         <v>4</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="16" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B3" s="16">
         <v>2</v>
@@ -4996,18 +5028,18 @@
     </row>
     <row r="4" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B4" s="16">
         <v>2</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="16" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B5" s="16">
         <v>0</v>
@@ -5030,7 +5062,7 @@
 </file>
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{252AC3CB-F2B0-42A6-9F5E-1AF0B499090D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C61EA33C-67F7-4189-8C73-ACBF9B808E17}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5040,13 +5072,13 @@
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -5057,7 +5089,7 @@
         <v>4</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -5077,7 +5109,7 @@
         <v>10</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -5105,7 +5137,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C183400A-0A99-4097-9646-65844BE42CE8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19780EC5-3F4E-4AAD-8BD9-7EE1D1BC76C1}">
   <dimension ref="A1:J40"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5118,23 +5150,23 @@
   <sheetData>
     <row r="1" spans="1:10" ht="44" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="4" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="J1" s="4" t="s">
         <v>8</v>
@@ -5142,7 +5174,7 @@
     </row>
     <row r="2" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B2" s="5">
         <v>4</v>
@@ -5160,7 +5192,7 @@
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="J2" s="7">
         <f>AVERAGE(Priklad!F2:F6)/(SQRT(Priklad!J14)^3)</f>
@@ -5169,7 +5201,7 @@
     </row>
     <row r="3" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B3" s="5">
         <v>2</v>
@@ -5187,7 +5219,7 @@
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
       <c r="I3" s="2" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="J3" s="7">
         <f>_xlfn.SKEW.P(Priklad!A2:A6)</f>
@@ -5196,7 +5228,7 @@
     </row>
     <row r="4" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B4" s="5">
         <v>2</v>
@@ -5214,7 +5246,7 @@
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
       <c r="I4" s="2" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="J4" s="7">
         <f>SKEW(Priklad!A2:A6)</f>
@@ -5223,7 +5255,7 @@
     </row>
     <row r="5" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B5" s="5">
         <v>0</v>
@@ -5241,7 +5273,7 @@
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
       <c r="I5" s="2" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="J5" s="7">
         <f>AVERAGE(Priklad!G2:G6)/(Priklad!J14^2)-3</f>
@@ -5258,7 +5290,7 @@
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
       <c r="I6" s="2" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="J6" s="7">
         <f>KURT(Priklad!A2:A6)</f>
@@ -5267,7 +5299,7 @@
     </row>
     <row r="7" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
@@ -5308,7 +5340,7 @@
     </row>
     <row r="10" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B10" s="14"/>
       <c r="C10" s="14"/>
@@ -5334,7 +5366,7 @@
     </row>
     <row r="12" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B12" s="14"/>
       <c r="C12" s="14"/>
@@ -5360,7 +5392,7 @@
     </row>
     <row r="14" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B14" s="14"/>
       <c r="C14" s="14"/>
@@ -5692,7 +5724,7 @@
     <mergeCell ref="A14:J14"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="whole" operator="greaterThanOrEqual" showInputMessage="1" sqref="B2:B5" xr:uid="{898EAEC6-915C-443A-A0DE-6195A9490D58}">
+    <dataValidation type="whole" operator="greaterThanOrEqual" showInputMessage="1" sqref="B2:B5" xr:uid="{30E57B9D-4C7B-4F91-A8B2-CA4C704DC5FB}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -5701,7 +5733,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{671192B0-BE21-46FA-85DF-D5FB6E645775}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{498BBBF5-E33D-45B7-A9F8-28F1DFBE773D}">
   <dimension ref="A1:J42"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5717,15 +5749,15 @@
   <sheetData>
     <row r="1" spans="1:10" ht="44" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="4" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="4" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="F1" s="1"/>
       <c r="G1" s="4" t="s">
@@ -5754,7 +5786,7 @@
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="2" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="H2" s="7">
         <f>_xlfn.PERCENTILE.INC(A2:A12,0.17)</f>
@@ -5780,7 +5812,7 @@
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="2" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="H3" s="7">
         <f>AVERAGE(C2:C11)</f>
@@ -5806,7 +5838,7 @@
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="2" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H4" s="7">
         <f>MEDIAN(C2:C11)</f>
@@ -5832,7 +5864,7 @@
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="2" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="H5" s="7">
         <f>_xlfn.PERCENTILE.INC(E2:E42,0.25)</f>
@@ -5858,7 +5890,7 @@
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="2" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="H6" s="7">
         <f>MEDIAN(E2:E42)</f>
@@ -5884,7 +5916,7 @@
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="2" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="H7" s="7">
         <f>_xlfn.PERCENTILE.INC(E2:E42,0.75)</f>
@@ -5910,7 +5942,7 @@
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="2" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="H8" s="7">
         <f>H7-H5</f>
@@ -5957,7 +5989,7 @@
       </c>
       <c r="F10" s="1"/>
       <c r="G10" s="13" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="H10" s="14"/>
       <c r="I10" s="1"/>
@@ -5998,7 +6030,7 @@
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="13" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="H12" s="14"/>
       <c r="I12" s="1"/>
@@ -6446,7 +6478,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F45CC14-CC14-4049-8FD3-8CE5B28489CD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA613495-794F-42FF-A36D-07952B397A68}">
   <dimension ref="A1:J40"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -6457,23 +6489,23 @@
   <sheetData>
     <row r="1" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="F1" s="1"/>
       <c r="G1" s="13" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="H1" s="14"/>
       <c r="I1" s="14"/>
@@ -6481,7 +6513,7 @@
     </row>
     <row r="2" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="B2" s="23">
         <v>6</v>
@@ -6490,7 +6522,7 @@
         <v>5</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E2" s="5">
         <v>2</v>
@@ -6503,7 +6535,7 @@
     </row>
     <row r="3" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="B3" s="23">
         <v>8</v>
@@ -6512,14 +6544,14 @@
         <v>9</v>
       </c>
       <c r="D3" s="20" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="E3" s="5">
         <v>4</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="13" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="H3" s="14"/>
       <c r="I3" s="14"/>
@@ -6527,7 +6559,7 @@
     </row>
     <row r="4" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="B4" s="23">
         <v>7</v>
@@ -6536,7 +6568,7 @@
         <v>8</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E4" s="5">
         <v>3</v>
@@ -6549,7 +6581,7 @@
     </row>
     <row r="5" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="B5" s="23">
         <v>5</v>
@@ -6558,14 +6590,14 @@
         <v>6</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="E5" s="5">
         <v>2</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="13" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="H5" s="14"/>
       <c r="I5" s="14"/>
@@ -6573,14 +6605,14 @@
     </row>
     <row r="6" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="B6" s="23"/>
       <c r="C6" s="5">
         <v>7</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E6" s="5">
         <v>3</v>
@@ -6593,7 +6625,7 @@
     </row>
     <row r="7" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="B7" s="23">
         <v>7</v>
@@ -6602,14 +6634,14 @@
         <v>0</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="E7" s="5">
         <v>1</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="13" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="H7" s="14"/>
       <c r="I7" s="14"/>
@@ -6617,7 +6649,7 @@
     </row>
     <row r="8" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B8" s="23">
         <v>4.5</v>
@@ -6626,7 +6658,7 @@
         <v>2</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="E8" s="5">
         <v>1</v>
@@ -6639,7 +6671,7 @@
     </row>
     <row r="9" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="B9" s="23">
         <v>6.3</v>
@@ -6648,14 +6680,14 @@
         <v>7</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E9" s="5">
         <v>3</v>
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="13" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="H9" s="14"/>
       <c r="I9" s="14"/>
@@ -6663,7 +6695,7 @@
     </row>
     <row r="10" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="B10" s="23">
         <v>7.3</v>
@@ -6672,7 +6704,7 @@
         <v>9</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E10" s="5">
         <v>4</v>
@@ -6685,7 +6717,7 @@
     </row>
     <row r="11" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="B11" s="23">
         <v>8.1</v>
@@ -6694,14 +6726,14 @@
         <v>4</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="E11" s="5">
         <v>2</v>
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="13" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="H11" s="14"/>
       <c r="I11" s="14"/>
@@ -6709,14 +6741,14 @@
     </row>
     <row r="12" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="B12" s="23"/>
       <c r="C12" s="5">
         <v>7</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E12" s="5">
         <v>3</v>
@@ -6729,7 +6761,7 @@
     </row>
     <row r="13" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="B13" s="23">
         <v>6</v>
@@ -6738,14 +6770,14 @@
         <v>10</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E13" s="5">
         <v>2</v>
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="13" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="H13" s="14"/>
       <c r="I13" s="14"/>
@@ -6753,7 +6785,7 @@
     </row>
     <row r="14" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="B14" s="23">
         <v>7.1</v>
@@ -6762,7 +6794,7 @@
         <v>5</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="E14" s="5">
         <v>3</v>
@@ -6775,7 +6807,7 @@
     </row>
     <row r="15" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="B15" s="23">
         <v>7.9</v>
@@ -6784,7 +6816,7 @@
         <v>8</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E15" s="5">
         <v>1</v>
@@ -6797,7 +6829,7 @@
     </row>
     <row r="16" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="B16" s="23">
         <v>9.1999999999999993</v>
@@ -6806,7 +6838,7 @@
         <v>11</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E16" s="5">
         <v>3</v>
@@ -6819,7 +6851,7 @@
     </row>
     <row r="17" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="B17" s="23">
         <v>5.5</v>
@@ -6828,7 +6860,7 @@
         <v>6</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="E17" s="5">
         <v>4</v>
@@ -6841,7 +6873,7 @@
     </row>
     <row r="18" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="B18" s="23">
         <v>6.8</v>
@@ -6850,7 +6882,7 @@
         <v>8</v>
       </c>
       <c r="D18" s="20" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E18" s="5">
         <v>2</v>
@@ -6863,7 +6895,7 @@
     </row>
     <row r="19" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="B19" s="23">
         <v>7.5</v>
@@ -6872,7 +6904,7 @@
         <v>3</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E19" s="5">
         <v>4</v>
@@ -6885,7 +6917,7 @@
     </row>
     <row r="20" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="B20" s="23">
         <v>8.8000000000000007</v>
@@ -6894,7 +6926,7 @@
         <v>7</v>
       </c>
       <c r="D20" s="20" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="E20" s="5">
         <v>2</v>
@@ -6907,7 +6939,7 @@
     </row>
     <row r="21" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="B21" s="23">
         <v>4.8</v>
@@ -6916,7 +6948,7 @@
         <v>9</v>
       </c>
       <c r="D21" s="20" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E21" s="5">
         <v>3</v>
@@ -6929,7 +6961,7 @@
     </row>
     <row r="22" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="B22" s="23">
         <v>6.5</v>
@@ -6938,7 +6970,7 @@
         <v>5</v>
       </c>
       <c r="D22" s="20" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E22" s="5">
         <v>1</v>
@@ -6951,7 +6983,7 @@
     </row>
     <row r="23" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="B23" s="23">
         <v>7.4</v>
@@ -6960,7 +6992,7 @@
         <v>7</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="E23" s="5">
         <v>3</v>
@@ -6973,7 +7005,7 @@
     </row>
     <row r="24" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="B24" s="23">
         <v>8.3000000000000007</v>
@@ -6982,7 +7014,7 @@
         <v>10</v>
       </c>
       <c r="D24" s="20" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E24" s="5">
         <v>4</v>
@@ -6995,14 +7027,14 @@
     </row>
     <row r="25" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="B25" s="23"/>
       <c r="C25" s="5">
         <v>6</v>
       </c>
       <c r="D25" s="20" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E25" s="5">
         <v>3</v>
@@ -7015,7 +7047,7 @@
     </row>
     <row r="26" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="B26" s="23">
         <v>6.2</v>
@@ -7024,7 +7056,7 @@
         <v>8</v>
       </c>
       <c r="D26" s="20" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="E26" s="5">
         <v>4</v>
@@ -7037,7 +7069,7 @@
     </row>
     <row r="27" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="B27" s="23">
         <v>7.2</v>
@@ -7046,7 +7078,7 @@
         <v>12</v>
       </c>
       <c r="D27" s="20" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E27" s="5">
         <v>2</v>
@@ -7059,7 +7091,7 @@
     </row>
     <row r="28" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="B28" s="23">
         <v>8</v>
@@ -7068,7 +7100,7 @@
         <v>6</v>
       </c>
       <c r="D28" s="20" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E28" s="5">
         <v>3</v>
@@ -7081,7 +7113,7 @@
     </row>
     <row r="29" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="B29" s="23">
         <v>9.5</v>
@@ -7090,7 +7122,7 @@
         <v>9</v>
       </c>
       <c r="D29" s="20" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="E29" s="5">
         <v>2</v>
@@ -7103,7 +7135,7 @@
     </row>
     <row r="30" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="B30" s="23">
         <v>5.8</v>
@@ -7112,7 +7144,7 @@
         <v>4</v>
       </c>
       <c r="D30" s="20" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E30" s="5">
         <v>3</v>
@@ -7125,7 +7157,7 @@
     </row>
     <row r="31" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="B31" s="23">
         <v>7</v>
@@ -7134,7 +7166,7 @@
         <v>7</v>
       </c>
       <c r="D31" s="20" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E31" s="5">
         <v>4</v>
@@ -7147,7 +7179,7 @@
     </row>
     <row r="32" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="B32" s="23">
         <v>7.7</v>
@@ -7156,7 +7188,7 @@
         <v>10</v>
       </c>
       <c r="D32" s="20" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="E32" s="5">
         <v>3</v>
@@ -7169,7 +7201,7 @@
     </row>
     <row r="33" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="B33" s="23">
         <v>9</v>
@@ -7178,7 +7210,7 @@
         <v>5</v>
       </c>
       <c r="D33" s="20" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E33" s="5">
         <v>4</v>
@@ -7191,7 +7223,7 @@
     </row>
     <row r="34" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="B34" s="23">
         <v>5.2</v>
@@ -7200,7 +7232,7 @@
         <v>8</v>
       </c>
       <c r="D34" s="20" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E34" s="5">
         <v>2</v>
@@ -7213,7 +7245,7 @@
     </row>
     <row r="35" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="B35" s="23">
         <v>6.5</v>
@@ -7222,7 +7254,7 @@
         <v>11</v>
       </c>
       <c r="D35" s="20" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="E35" s="5">
         <v>3</v>
@@ -7235,7 +7267,7 @@
     </row>
     <row r="36" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="B36" s="23">
         <v>7.5</v>
@@ -7244,7 +7276,7 @@
         <v>6</v>
       </c>
       <c r="D36" s="20" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E36" s="5">
         <v>2</v>
@@ -7257,7 +7289,7 @@
     </row>
     <row r="37" spans="1:10" ht="22.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="B37" s="23">
         <v>8.5</v>
@@ -7266,7 +7298,7 @@
         <v>8</v>
       </c>
       <c r="D37" s="20" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E37" s="5">
         <v>3</v>
@@ -7328,7 +7360,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1753A032-2588-4CA5-9429-EF10BD63D566}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94104B57-8D0F-465D-B5EA-87EB75155984}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -7341,7 +7373,7 @@
         <v>0</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -7349,7 +7381,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -7363,7 +7395,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -7391,7 +7423,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7266524D-3FF4-4F6D-8E64-D2AB9AD15E47}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AA817B3-5704-4A58-BBDC-5E9AE1D5378E}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -7401,13 +7433,13 @@
   <sheetData>
     <row r="1" spans="1:4" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D1" s="17" t="s">
         <v>78</v>
-      </c>
-      <c r="D1" s="17" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -7418,7 +7450,7 @@
         <v>2</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -7438,7 +7470,7 @@
         <v>6</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -7472,7 +7504,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82E5FF3B-C65D-4BCF-ADBF-75F2DD75DB91}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E729BF0D-C737-4EAE-A9F2-DF2E52C99CE4}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -7482,10 +7514,10 @@
   <sheetData>
     <row r="1" spans="1:3" ht="46.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -7493,7 +7525,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">
@@ -7507,7 +7539,7 @@
         <v>6</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>